<commit_message>
Update Tennessee proposal and map data
</commit_message>
<xml_diff>
--- a/TN/dataset/tennessee_public_data_centers.xlsx
+++ b/TN/dataset/tennessee_public_data_centers.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rf9d9800af38a4a03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R3574101214004509"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master" sheetId="3" r:id="R5082f2aa05f24078"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw_Aligned" sheetId="4" r:id="Ra9cfb7e8060e46dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Match_Audit" sheetId="5" r:id="R23c9e5d603d24ef3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Pairs" sheetId="6" r:id="R1b39ba1c1ad440e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded_Support" sheetId="7" r:id="R50f1835ae13d4a7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field_Map" sheetId="8" r:id="Rf51c3b862c0f44bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidate_Sites" sheetId="9" r:id="R251ed96a6c2f4629"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Log" sheetId="10" r:id="R733927bef93b4ac9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proposal_Readiness" sheetId="11" r:id="R1f6490a475fc4beb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Queue" sheetId="12" r:id="Ree55e08506e54a19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Location_Audit" sheetId="13" r:id="Rb96916fd01d84047"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R0d2aded890494020"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R1cc297d0f7004afc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master" sheetId="3" r:id="R5813bdeb2eac46ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw_Aligned" sheetId="4" r:id="R3b25501127854222"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Match_Audit" sheetId="5" r:id="Rd134fd093d564f31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Pairs" sheetId="6" r:id="R2090a52bcc934526"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded_Support" sheetId="7" r:id="Rf5dfaf003577423a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field_Map" sheetId="8" r:id="Rbd0d0e93089f4341"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidate_Sites" sheetId="9" r:id="R016acd8d38e047c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Log" sheetId="10" r:id="R226e36a77a544718"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proposal_Readiness" sheetId="11" r:id="R1acf0415faed407e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Queue" sheetId="12" r:id="Rcd08d83c01af4cd3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Location_Audit" sheetId="13" r:id="Rf58b1f9db49d44a3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1383,7 +1383,7 @@
         <x:v>Verification policy</x:v>
       </x:c>
       <x:c r="B22" s="85" t="str">
-        <x:v>2026-09-04 fifth-pass candidate-location research: Jackson physical street address resolved to 2342 North Parkway East via JEA + SEC ownership chain; Atmosphere receives only a low-confidence market pin, explicitly not the 38-acre parcel; Mountain City parcel identity is high-confidence but WGS84 remains unresolved; Scipio remains explicitly non-public.</x:v>
+        <x:v>2026-09-07 review-queue resolution: Cielo remains in Master only for source traceability with analysis_scope=unconfirmed_candidate and is excluded from confirmed spatial training; the Atmosphere market pin was removed; linked and address discrepancies are documented in Review_Queue and model/data/metadata/review_queue_research_ledger.csv.</x:v>
       </x:c>
       <x:c r="C22" s="85" t="str">
         <x:v>Uncertain status, scope, or identity stays in Candidate_Sites</x:v>
@@ -4742,6 +4742,292 @@
         <x:v>Parcel identity strengthened; no textual WGS84 point found.</x:v>
       </x:c>
     </x:row>
+    <x:row r="135">
+      <x:c r="A135" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="B135" t="str">
+        <x:v>TNDC-006</x:v>
+      </x:c>
+      <x:c r="C135" t="str">
+        <x:v>UPDATE</x:v>
+      </x:c>
+      <x:c r="D135" t="str">
+        <x:v>analysis_scope</x:v>
+      </x:c>
+      <x:c r="E135" t="str">
+        <x:v>core_data_center</x:v>
+      </x:c>
+      <x:c r="F135" t="str">
+        <x:v>unconfirmed_candidate</x:v>
+      </x:c>
+      <x:c r="G135" t="str">
+        <x:v>../model/data/metadata/review_queue_research_ledger.csv</x:v>
+      </x:c>
+      <x:c r="H135" t="str">
+        <x:v>Local reporting conflicts with market listings; retain traceability but exclude from confirmed spatial presence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136">
+      <x:c r="A136" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="B136" t="str">
+        <x:v>TNDC-023</x:v>
+      </x:c>
+      <x:c r="C136" t="str">
+        <x:v>UPDATE</x:v>
+      </x:c>
+      <x:c r="D136" t="str">
+        <x:v>verification_note</x:v>
+      </x:c>
+      <x:c r="E136" t="str">
+        <x:v>Local vicinity note</x:v>
+      </x:c>
+      <x:c r="F136" t="str">
+        <x:v>Approximate-vicinity decision</x:v>
+      </x:c>
+      <x:c r="G136" t="str">
+        <x:v>../model/data/metadata/review_queue_research_ledger.csv</x:v>
+      </x:c>
+      <x:c r="H136" t="str">
+        <x:v>Official developer page lacks a parcel; prevent false exact-site interpretation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137">
+      <x:c r="A137" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="B137" t="str">
+        <x:v>Retired TNDC-025</x:v>
+      </x:c>
+      <x:c r="C137" t="str">
+        <x:v>UPDATE</x:v>
+      </x:c>
+      <x:c r="D137" t="str">
+        <x:v>Review_Pairs rationale</x:v>
+      </x:c>
+      <x:c r="E137" t="str">
+        <x:v>blank</x:v>
+      </x:c>
+      <x:c r="F137" t="str">
+        <x:v>No forced Colossus merge</x:v>
+      </x:c>
+      <x:c r="G137" t="str">
+        <x:v>../model/data/metadata/review_queue_research_ledger.csv</x:v>
+      </x:c>
+      <x:c r="H137" t="str">
+        <x:v>Generic source cannot be assigned safely to either xAI campus.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138">
+      <x:c r="A138" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="B138" t="str">
+        <x:v>TNDC-037</x:v>
+      </x:c>
+      <x:c r="C138" t="str">
+        <x:v>UPDATE</x:v>
+      </x:c>
+      <x:c r="D138" t="str">
+        <x:v>address</x:v>
+      </x:c>
+      <x:c r="E138" t="str">
+        <x:v>2992 Sidco Drive</x:v>
+      </x:c>
+      <x:c r="F138" t="str">
+        <x:v>2990 Sidco Drive</x:v>
+      </x:c>
+      <x:c r="G138" t="str">
+        <x:v>../model/data/metadata/review_queue_research_ledger.csv</x:v>
+      </x:c>
+      <x:c r="H138" t="str">
+        <x:v>Use current Lumen route-list address; retain legacy discrepancy in note.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139">
+      <x:c r="A139" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="B139" t="str">
+        <x:v>TNDC-039</x:v>
+      </x:c>
+      <x:c r="C139" t="str">
+        <x:v>UPDATE</x:v>
+      </x:c>
+      <x:c r="D139" t="str">
+        <x:v>operator</x:v>
+      </x:c>
+      <x:c r="E139" t="str">
+        <x:v>Fisk University</x:v>
+      </x:c>
+      <x:c r="F139" t="str">
+        <x:v>blank; Fisk retained as project sponsor</x:v>
+      </x:c>
+      <x:c r="G139" t="str">
+        <x:v>../model/data/metadata/review_queue_research_ledger.csv</x:v>
+      </x:c>
+      <x:c r="H139" t="str">
+        <x:v>Operating partner is not publicly identified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140">
+      <x:c r="A140" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="B140" t="str">
+        <x:v>TNDC-002|TNDC-009</x:v>
+      </x:c>
+      <x:c r="C140" t="str">
+        <x:v>UPDATE</x:v>
+      </x:c>
+      <x:c r="D140" t="str">
+        <x:v>facility mapping</x:v>
+      </x:c>
+      <x:c r="E140" t="str">
+        <x:v>queue ambiguity</x:v>
+      </x:c>
+      <x:c r="F140" t="str">
+        <x:v>two distinct SEC-mapped properties</x:v>
+      </x:c>
+      <x:c r="G140" t="str">
+        <x:v>../model/data/metadata/review_queue_research_ledger.csv</x:v>
+      </x:c>
+      <x:c r="H140" t="str">
+        <x:v>SEC evidence confirms both Crossville addresses and no merge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141">
+      <x:c r="A141" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="B141" t="str">
+        <x:v>TNDC-059</x:v>
+      </x:c>
+      <x:c r="C141" t="str">
+        <x:v>UPDATE</x:v>
+      </x:c>
+      <x:c r="D141" t="str">
+        <x:v>verification_class</x:v>
+      </x:c>
+      <x:c r="E141" t="str">
+        <x:v>review</x:v>
+      </x:c>
+      <x:c r="F141" t="str">
+        <x:v>confirmed</x:v>
+      </x:c>
+      <x:c r="G141" t="str">
+        <x:v>../model/data/metadata/review_queue_research_ledger.csv</x:v>
+      </x:c>
+      <x:c r="H141" t="str">
+        <x:v>Facility-facing 4280 address and broader-site 4300 permit address are explicitly distinguished.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142">
+      <x:c r="A142" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="B142" t="str">
+        <x:v>TNCAND-005</x:v>
+      </x:c>
+      <x:c r="C142" t="str">
+        <x:v>UPDATE</x:v>
+      </x:c>
+      <x:c r="D142" t="str">
+        <x:v>review_note</x:v>
+      </x:c>
+      <x:c r="E142" t="str">
+        <x:v>prior note</x:v>
+      </x:c>
+      <x:c r="F142" t="str">
+        <x:v>current evidence limit recorded</x:v>
+      </x:c>
+      <x:c r="G142" t="str">
+        <x:v>../model/data/metadata/review_queue_research_ledger.csv</x:v>
+      </x:c>
+      <x:c r="H142" t="str">
+        <x:v>Not promoted without current operating confirmation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143">
+      <x:c r="A143" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="B143" t="str">
+        <x:v>TNCAND-006</x:v>
+      </x:c>
+      <x:c r="C143" t="str">
+        <x:v>UPDATE</x:v>
+      </x:c>
+      <x:c r="D143" t="str">
+        <x:v>latitude|longitude</x:v>
+      </x:c>
+      <x:c r="E143" t="str">
+        <x:v>market pin</x:v>
+      </x:c>
+      <x:c r="F143" t="str">
+        <x:v>blank</x:v>
+      </x:c>
+      <x:c r="G143" t="str">
+        <x:v>../model/data/metadata/review_queue_research_ledger.csv</x:v>
+      </x:c>
+      <x:c r="H143" t="str">
+        <x:v>No public parcel; remove physically inconsistent point from spatial use.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144">
+      <x:c r="A144" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="B144" t="str">
+        <x:v>TNCAND-012</x:v>
+      </x:c>
+      <x:c r="C144" t="str">
+        <x:v>UPDATE</x:v>
+      </x:c>
+      <x:c r="D144" t="str">
+        <x:v>candidate_type</x:v>
+      </x:c>
+      <x:c r="E144" t="str">
+        <x:v>unresolved_duplicate_or_new_facility</x:v>
+      </x:c>
+      <x:c r="F144" t="str">
+        <x:v>linked_master_evidence</x:v>
+      </x:c>
+      <x:c r="G144" t="str">
+        <x:v>../model/data/metadata/review_queue_research_ledger.csv</x:v>
+      </x:c>
+      <x:c r="H144" t="str">
+        <x:v>Shared address links this evidence to TNDC-038.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145">
+      <x:c r="A145" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="B145" t="str">
+        <x:v>TNCAND-013–016</x:v>
+      </x:c>
+      <x:c r="C145" t="str">
+        <x:v>UPDATE</x:v>
+      </x:c>
+      <x:c r="D145" t="str">
+        <x:v>review_note</x:v>
+      </x:c>
+      <x:c r="E145" t="str">
+        <x:v>legacy status unclear</x:v>
+      </x:c>
+      <x:c r="F145" t="str">
+        <x:v>primary-evidence requirement recorded</x:v>
+      </x:c>
+      <x:c r="G145" t="str">
+        <x:v>../model/data/metadata/review_queue_research_ledger.csv</x:v>
+      </x:c>
+      <x:c r="H145" t="str">
+        <x:v>Retained as candidates; do not promote from directory evidence alone.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -5090,19 +5376,19 @@
         <x:v>Cielo Montgomery County AI Campus</x:v>
       </x:c>
       <x:c r="C2" s="85" t="str">
-        <x:v>verification</x:v>
+        <x:v>closed_with_evidence</x:v>
       </x:c>
       <x:c r="D2" s="85" t="str">
-        <x:v>Candidate/unverified market listing; local June 2026 reporting said no data-center proposal was under discussion.</x:v>
+        <x:v>Resolved in 2026-09-07 review: TNDC-006</x:v>
       </x:c>
       <x:c r="E2" s="85" t="str">
-        <x:v>Keep as candidate; do not use as confirmed treatment unless new local evidence appears.</x:v>
+        <x:v>No open action for this dataset version. Evidence and disposition: ../model/data/metadata/review_queue_research_ledger.csv</x:v>
       </x:c>
       <x:c r="F2" s="85" t="str">
         <x:v>multiple public sources; local contradiction</x:v>
       </x:c>
       <x:c r="G2" s="85" t="str">
-        <x:v>high</x:v>
+        <x:v>closed</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -5113,19 +5399,19 @@
         <x:v>Hixson Data Center (McMinnville)</x:v>
       </x:c>
       <x:c r="C3" s="85" t="str">
-        <x:v>coordinate</x:v>
+        <x:v>closed_with_evidence</x:v>
       </x:c>
       <x:c r="D3" s="85" t="str">
-        <x:v>Coordinate disagreement exceeds 7 km; only area/city-level point is defensible.</x:v>
+        <x:v>Resolved in 2026-09-07 review: TNDC-023</x:v>
       </x:c>
       <x:c r="E3" s="85" t="str">
-        <x:v>Resolve parcel/site before parcel-distance analysis.</x:v>
+        <x:v>No open action for this dataset version. Evidence and disposition: ../model/data/metadata/review_queue_research_ledger.csv</x:v>
       </x:c>
       <x:c r="F3" s="85" t="str">
         <x:v>source coordinate conflict retained</x:v>
       </x:c>
       <x:c r="G3" s="85" t="str">
-        <x:v>high</x:v>
+        <x:v>closed</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -5136,19 +5422,19 @@
         <x:v>Generic Colossus source identity</x:v>
       </x:c>
       <x:c r="C4" s="85" t="str">
-        <x:v>entity_resolution_retired</x:v>
+        <x:v>closed_with_evidence</x:v>
       </x:c>
       <x:c r="D4" s="85" t="str">
-        <x:v>Removed from Master because it necessarily overlaps TNDC-030 or TNDC-031 but cannot be assigned safely.</x:v>
+        <x:v>Resolved in 2026-09-07 review: Retired TNDC-025</x:v>
       </x:c>
       <x:c r="E4" s="85" t="str">
-        <x:v>Resolve only if new source evidence identifies the matching campus; otherwise retain in Raw_Aligned and Review_Pairs.</x:v>
+        <x:v>No open action for this dataset version. Evidence and disposition: ../model/data/metadata/review_queue_research_ledger.csv</x:v>
       </x:c>
       <x:c r="F4" s="85" t="str">
         <x:v>all source records and URLs retained</x:v>
       </x:c>
       <x:c r="G4" s="85" t="str">
-        <x:v>high</x:v>
+        <x:v>closed</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -5159,19 +5445,19 @@
         <x:v>Level(3)/Lumen Nashville (Sidco)</x:v>
       </x:c>
       <x:c r="C5" s="85" t="str">
-        <x:v>address</x:v>
+        <x:v>closed_with_evidence</x:v>
       </x:c>
       <x:c r="D5" s="85" t="str">
-        <x:v>Master has 2992 Sidco Drive while independent confirmed list reports 2990 Sidco Drive.</x:v>
+        <x:v>Resolved in 2026-09-07 review: TNDC-037</x:v>
       </x:c>
       <x:c r="E5" s="85" t="str">
-        <x:v>Resolve parcel/address before exact geospatial joins.</x:v>
+        <x:v>No open action for this dataset version. Evidence and disposition: ../model/data/metadata/review_queue_research_ledger.csv</x:v>
       </x:c>
       <x:c r="F5" s="85" t="str">
         <x:v>address contradiction</x:v>
       </x:c>
       <x:c r="G5" s="85" t="str">
-        <x:v>medium</x:v>
+        <x:v>closed</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -5182,19 +5468,19 @@
         <x:v>Quantum Leap Data Center / Fisk University</x:v>
       </x:c>
       <x:c r="C6" s="85" t="str">
-        <x:v>operator</x:v>
+        <x:v>closed_with_evidence</x:v>
       </x:c>
       <x:c r="D6" s="85" t="str">
-        <x:v>Fisk confirms project/campus but operating data-center partner is not publicly identified.</x:v>
+        <x:v>Resolved in 2026-09-07 review: TNDC-039</x:v>
       </x:c>
       <x:c r="E6" s="85" t="str">
-        <x:v>Leave operator null until public operator evidence exists.</x:v>
+        <x:v>No open action for this dataset version. Evidence and disposition: ../model/data/metadata/review_queue_research_ledger.csv</x:v>
       </x:c>
       <x:c r="F6" s="85" t="str">
         <x:v>project verified; operator unresolved</x:v>
       </x:c>
       <x:c r="G6" s="85" t="str">
-        <x:v>medium</x:v>
+        <x:v>closed</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -5205,19 +5491,19 @@
         <x:v>CleanSpark Crossville pair</x:v>
       </x:c>
       <x:c r="C7" s="85" t="str">
-        <x:v>address</x:v>
+        <x:v>closed_with_evidence</x:v>
       </x:c>
       <x:c r="D7" s="85" t="str">
-        <x:v>Two public Crossville addresses cannot be reliably assigned to TNDC-002 versus TNDC-009.</x:v>
+        <x:v>Resolved in 2026-09-07 review: TNDC-002</x:v>
       </x:c>
       <x:c r="E7" s="85" t="str">
-        <x:v>Leave both Master addresses null until facility-name mapping is sourced.</x:v>
+        <x:v>No open action for this dataset version. Evidence and disposition: ../model/data/metadata/review_queue_research_ledger.csv</x:v>
       </x:c>
       <x:c r="F7" s="85" t="str">
         <x:v>DataCenterMap market page retained in both records</x:v>
       </x:c>
       <x:c r="G7" s="85" t="str">
-        <x:v>high</x:v>
+        <x:v>closed</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -5228,19 +5514,19 @@
         <x:v>5C MEM01</x:v>
       </x:c>
       <x:c r="C8" s="85" t="str">
-        <x:v>address</x:v>
+        <x:v>closed_with_evidence</x:v>
       </x:c>
       <x:c r="D8" s="85" t="str">
-        <x:v>County/public-health records use 4300 Getwell Rd; some directories use 4280 Getwell Rd.</x:v>
+        <x:v>Resolved in 2026-09-07 review: TNDC-059</x:v>
       </x:c>
       <x:c r="E8" s="85" t="str">
-        <x:v>Use 4300 as the official public-record address and retain the discrepancy.</x:v>
+        <x:v>No open action for this dataset version. Evidence and disposition: ../model/data/metadata/review_queue_research_ledger.csv</x:v>
       </x:c>
       <x:c r="F8" s="85" t="str">
         <x:v>official and industry sources retained</x:v>
       </x:c>
       <x:c r="G8" s="85" t="str">
-        <x:v>medium</x:v>
+        <x:v>closed</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -5251,19 +5537,19 @@
         <x:v>GRIID Jackson 60 MW Project</x:v>
       </x:c>
       <x:c r="C9" s="85" t="str">
-        <x:v>project_status</x:v>
+        <x:v>closed_with_evidence</x:v>
       </x:c>
       <x:c r="D9" s="85" t="str">
-        <x:v>Announcement predates CleanSpark acquisition; no current site-level confirmation found.</x:v>
+        <x:v>Resolved in 2026-09-07 review: TNCAND-005</x:v>
       </x:c>
       <x:c r="E9" s="85" t="str">
-        <x:v>Do not promote until parcel and current status are confirmed.</x:v>
+        <x:v>No open action for this dataset version. Evidence and disposition: ../model/data/metadata/review_queue_research_ledger.csv</x:v>
       </x:c>
       <x:c r="F9" s="85" t="str">
         <x:v>announcement, acquisition, and SEC records retained</x:v>
       </x:c>
       <x:c r="G9" s="85" t="str">
-        <x:v>high</x:v>
+        <x:v>closed</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -5274,19 +5560,19 @@
         <x:v>Atmosphere Nashville Campus</x:v>
       </x:c>
       <x:c r="C10" s="85" t="str">
-        <x:v>location</x:v>
+        <x:v>closed_with_evidence</x:v>
       </x:c>
       <x:c r="D10" s="85" t="str">
-        <x:v>Developer discloses scale but not an exact site.</x:v>
+        <x:v>Resolved in 2026-09-07 review: TNCAND-006</x:v>
       </x:c>
       <x:c r="E10" s="85" t="str">
-        <x:v>Keep as candidate until permitting or parcel evidence appears.</x:v>
+        <x:v>No open action for this dataset version. Evidence and disposition: ../model/data/metadata/review_queue_research_ledger.csv</x:v>
       </x:c>
       <x:c r="F10" s="85" t="str">
         <x:v>developer and trade reporting retained</x:v>
       </x:c>
       <x:c r="G10" s="85" t="str">
-        <x:v>high</x:v>
+        <x:v>closed</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -5297,19 +5583,19 @@
         <x:v>Scipio NREP Listing</x:v>
       </x:c>
       <x:c r="C11" s="85" t="str">
-        <x:v>entity_resolution</x:v>
+        <x:v>closed_with_evidence</x:v>
       </x:c>
       <x:c r="D11" s="85" t="str">
-        <x:v>Could be TNDC-038 or a distinct Nashville site.</x:v>
+        <x:v>Resolved in 2026-09-07 review: TNCAND-012</x:v>
       </x:c>
       <x:c r="E11" s="85" t="str">
-        <x:v>Do not create another Master row without a distinct street address.</x:v>
+        <x:v>No open action for this dataset version. Evidence and disposition: ../model/data/metadata/review_queue_research_ledger.csv</x:v>
       </x:c>
       <x:c r="F11" s="85" t="str">
         <x:v>market directory and operator support page retained</x:v>
       </x:c>
       <x:c r="G11" s="85" t="str">
-        <x:v>high</x:v>
+        <x:v>closed</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -5320,19 +5606,19 @@
         <x:v>Legacy operational listings</x:v>
       </x:c>
       <x:c r="C12" s="85" t="str">
-        <x:v>current_status</x:v>
+        <x:v>closed_with_evidence</x:v>
       </x:c>
       <x:c r="D12" s="85" t="str">
-        <x:v>Historic/current directories identify physical sites, but present data-center operations are not explicit enough.</x:v>
+        <x:v>Resolved in 2026-09-07 review: TNCAND-013–016</x:v>
       </x:c>
       <x:c r="E12" s="85" t="str">
-        <x:v>Confirm current operator service before promotion to Master.</x:v>
+        <x:v>No open action for this dataset version. Evidence and disposition: ../model/data/metadata/review_queue_research_ledger.csv</x:v>
       </x:c>
       <x:c r="F12" s="85" t="str">
         <x:v>all supporting URLs retained in Candidate_Sites</x:v>
       </x:c>
       <x:c r="G12" s="85" t="str">
-        <x:v>medium</x:v>
+        <x:v>closed</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5603,13 +5889,13 @@
         <x:v>low</x:v>
       </x:c>
       <x:c r="J7" s="85" t="str">
-        <x:v>address | postal_code</x:v>
+        <x:v>unconfirmed_project_and_exact_site</x:v>
       </x:c>
       <x:c r="K7" s="85" t="str">
-        <x:v>COMPLIANT_PARTIAL</x:v>
+        <x:v>EXCLUDED_UNCONFIRMED</x:v>
       </x:c>
       <x:c r="L7" s="85" t="str">
-        <x:v>Coordinate populated with explicit non-exact precision/confidence and provenance.</x:v>
+        <x:v>Cielo is retained for source traceability only; local reporting conflicts with market listings. Excluded from confirmed spatial presence.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -6216,12 +6502,14 @@
       <x:c r="I24" s="85" t="str">
         <x:v>medium</x:v>
       </x:c>
-      <x:c r="J24" s="85" t="str"/>
+      <x:c r="J24" s="85" t="str">
+        <x:v>exact_parcel</x:v>
+      </x:c>
       <x:c r="K24" s="85" t="str">
-        <x:v>COMPLIANT_PARTIAL</x:v>
+        <x:v>APPROXIMATE_VICINITY</x:v>
       </x:c>
       <x:c r="L24" s="85" t="str">
-        <x:v>Coordinate populated with explicit non-exact precision/confidence and provenance.</x:v>
+        <x:v>Hixson confirms McMinnville/Warren County but has not published a parcel. 191 Industrial Dr is a local-reporting vicinity only.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -6670,7 +6958,7 @@
         <x:v>Nashville</x:v>
       </x:c>
       <x:c r="E37" s="85" t="str">
-        <x:v>2992 Sidco Drive</x:v>
+        <x:v>2990 Sidco Drive</x:v>
       </x:c>
       <x:c r="F37" s="85" t="n">
         <x:v>36.102726</x:v>
@@ -6686,10 +6974,10 @@
       </x:c>
       <x:c r="J37" s="85" t="str"/>
       <x:c r="K37" s="85" t="str">
-        <x:v>RESOLVED</x:v>
+        <x:v>ADDRESS_CANONICALIZED</x:v>
       </x:c>
       <x:c r="L37" s="85" t="str">
-        <x:v>Address/site-level location fully populated at high confidence.</x:v>
+        <x:v>Lumen current route list uses 2990 Sidco Drive; 2992 is retained as an adjacent legacy-directory discrepancy.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -7478,10 +7766,10 @@
       </x:c>
       <x:c r="J59" s="85" t="str"/>
       <x:c r="K59" s="85" t="str">
-        <x:v>COMPLIANT_PARTIAL</x:v>
+        <x:v>ADDRESS_CONTEXT_RESOLVED</x:v>
       </x:c>
       <x:c r="L59" s="85" t="str">
-        <x:v>Coordinate populated with explicit non-exact precision/confidence and provenance.</x:v>
+        <x:v>4280 Getwell Rd remains the facility-facing address; 4300 Getwell Rd is related broader-site permit/property evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -7748,12 +8036,8 @@
         <x:v>Nashville</x:v>
       </x:c>
       <x:c r="E67" s="85"/>
-      <x:c r="F67" s="85" t="n">
-        <x:v>36.16488198</x:v>
-      </x:c>
-      <x:c r="G67" s="85" t="n">
-        <x:v>-86.78088767</x:v>
-      </x:c>
+      <x:c r="F67" s="85" t="str"/>
+      <x:c r="G67" s="85" t="str"/>
       <x:c r="H67" s="85" t="str">
         <x:v>area_or_city</x:v>
       </x:c>
@@ -7761,13 +8045,13 @@
         <x:v>low</x:v>
       </x:c>
       <x:c r="J67" s="85" t="str">
-        <x:v>address | county | postal_code</x:v>
+        <x:v>exact_site|latitude|longitude</x:v>
       </x:c>
       <x:c r="K67" s="85" t="str">
-        <x:v>MARKET_PIN_ONLY</x:v>
+        <x:v>MARKET_ONLY</x:v>
       </x:c>
       <x:c r="L67" s="85" t="str">
-        <x:v>Coordinate is a low-confidence directory/market pin and must not be used as the 38-acre campus parcel.</x:v>
+        <x:v>Developer discloses Nashville project but no site. Removed the physically inconsistent market pin from spatial use.</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -7963,23 +8247,25 @@
       <x:c r="D73" s="85" t="str">
         <x:v>Nashville</x:v>
       </x:c>
-      <x:c r="E73" s="85"/>
+      <x:c r="E73" s="85" t="str">
+        <x:v>1661 Murfreesboro Pike</x:v>
+      </x:c>
       <x:c r="F73" s="85"/>
       <x:c r="G73" s="85"/>
       <x:c r="H73" s="85" t="str">
-        <x:v>area_or_city</x:v>
+        <x:v>address_or_site</x:v>
       </x:c>
       <x:c r="I73" s="85" t="str">
-        <x:v>low</x:v>
+        <x:v>high</x:v>
       </x:c>
       <x:c r="J73" s="85" t="str">
-        <x:v>address | latitude | longitude</x:v>
+        <x:v>none_linked_duplicate</x:v>
       </x:c>
       <x:c r="K73" s="85" t="str">
-        <x:v>EXPLICIT_NON_PUBLIC</x:v>
+        <x:v>LINKED_TO_MASTER</x:v>
       </x:c>
       <x:c r="L73" s="85" t="str">
-        <x:v>Current facility directory explicitly states the exact location is not public.</x:v>
+        <x:v>Shared public address links Scipio evidence to TNDC-038; not a distinct facility point.</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -8287,7 +8573,7 @@
       </x:c>
       <x:c r="B7" s="131" t="n">
         <x:f>COUNTIF(Master!V2:V1000,"core_data_center")</x:f>
-        <x:v>50</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="C7" s="67" t="str">
         <x:v>50 core entities after adding the independently verified Bristol facility; building-level records within existing campuses remain deduplicated.</x:v>
@@ -8422,7 +8708,7 @@
       </x:c>
       <x:c r="B13" s="131" t="n">
         <x:f>COUNTBLANK('Master'!C2:C61)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C13" s="67" t="str">
         <x:v>Missing operators have explicit operator_status; unknown values are not fabricated.</x:v>
@@ -8824,7 +9110,7 @@
         <x:v>https://www.prnewswire.com/news-releases/cleanspark-to-add-5-ehs-and-increase-2024-guidance-with-acquisition-of-seven-additional-bitcoin-mining-facilities-in-tennessee-302244673.html | https://www.sec.gov/Archives/edgar/data/827876/000119312525297510/clsk-20250930.htm | https://www.datacentermap.com/usa/tennessee/crossville/ | https://www.sec.gov/Archives/edgar/data/827876/000095017024105354/clsk-ex10_4.htm</x:v>
       </x:c>
       <x:c r="AF3" s="128" t="str">
-        <x:v>2026-09-04</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="AG3" s="85" t="str">
         <x:v>confirmed</x:v>
@@ -8845,7 +9131,7 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="AM3" s="85" t="str">
-        <x:v>SEC filing identifies the Campbell Junction Property at this address; existing approximate GPS retained.</x:v>
+        <x:v>CleanSpark SEC evidence maps Campbell Junction Property to 5784 Plateau Rd. The separate West Crossville property is 268 Sparta Hwy (TNDC-009); retain two facilities and do not merge.</x:v>
       </x:c>
       <x:c r="AN3" s="85" t="str">
         <x:v>1.1</x:v>
@@ -9264,7 +9550,7 @@
         <x:v>data_center</x:v>
       </x:c>
       <x:c r="V7" s="17" t="str">
-        <x:v>core_data_center</x:v>
+        <x:v>unconfirmed_candidate</x:v>
       </x:c>
       <x:c r="W7" s="91" t="n">
         <x:v>350</x:v>
@@ -9275,7 +9561,7 @@
       </x:c>
       <x:c r="Z7" s="35"/>
       <x:c r="AA7" s="17" t="str">
-        <x:v>compute_atlas | fractracker | server_country | datacenterwatch | fractracker_arcgis | servercountry.org | datacenterwatch.ai | services1.arcgis.com</x:v>
+        <x:v>compute_atlas | fractracker | server_country | datacenterwatch | fractracker_arcgis | servercountry.org | datacenterwatch.ai | services1.arcgis.com | clarksvillenow</x:v>
       </x:c>
       <x:c r="AB7" s="94" t="n">
         <x:v>8</x:v>
@@ -9287,10 +9573,10 @@
         <x:v>compute_atlas:cielo-clarksville-tn | fractracker:495</x:v>
       </x:c>
       <x:c r="AE7" s="23" t="str">
-        <x:v>https://cieloinfra.com/ | https://cleanview.co/data-centers/tennessee/2037/cielo-clarksville-data-center | https://www.arcgis.com/home/item.html?id=597555ce8e4a4892a030784a7c657fdd | https://www.datacenterdynamics.com/en/news/cielo-digital-infrastructure-plans-300mw-data-center-campus-in-south-carolina/ | https://www.servercountry.org/policy/tennessee/ | https://datacenterwatch.ai/proposals/fractracker-tn-unknown-operator-cielo-digital-infrastructure-686 | https://services1.arcgis.com/4yjifSiIG17X0gW4/arcgis/rest/services/Data_Centers/FeatureServer/0/query?where=OBJECTID%3D5239&amp;outFields=*&amp;returnGeometry=true&amp;f=json | https://registry.deploy.report/datacenters/facilities/cielo-clarksville-data-center-tn</x:v>
+        <x:v>https://cieloinfra.com/ | https://cleanview.co/data-centers/tennessee/2037/cielo-clarksville-data-center | https://www.arcgis.com/home/item.html?id=597555ce8e4a4892a030784a7c657fdd | https://www.datacenterdynamics.com/en/news/cielo-digital-infrastructure-plans-300mw-data-center-campus-in-south-carolina/ | https://www.servercountry.org/policy/tennessee/ | https://datacenterwatch.ai/proposals/fractracker-tn-unknown-operator-cielo-digital-infrastructure-686 | https://services1.arcgis.com/4yjifSiIG17X0gW4/arcgis/rest/services/Data_Centers/FeatureServer/0/query?where=OBJECTID%3D5239&amp;outFields=*&amp;returnGeometry=true&amp;f=json | https://registry.deploy.report/datacenters/facilities/cielo-clarksville-data-center-tn | https://clarksvillenow.com/local/council-discusses-data-center-concerns-but-no-proposal-is-on-the-table/</x:v>
       </x:c>
       <x:c r="AF7" s="128" t="str">
-        <x:v>2026-09-04</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="AG7" s="85" t="str">
         <x:v>candidate</x:v>
@@ -9305,13 +9591,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AK7" s="96" t="n">
-        <x:v>75</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AL7" s="85" t="str">
-        <x:v>medium</x:v>
+        <x:v>low</x:v>
       </x:c>
       <x:c r="AM7" s="85" t="str">
-        <x:v>Current reviewed sources support Clarksville/Montgomery County but no public parcel/street address; broad coordinate is intentionally area_or_city / low.</x:v>
+        <x:v>Public market directories list a planned 350 MW Clarksville project, while June 2026 local reporting said the planning commission had no proposal under discussion. No primary local filing was identified. Retained for source traceability only as an unconfirmed candidate and excluded from confirmed-presence spatial training.</x:v>
       </x:c>
       <x:c r="AN7" s="85" t="str">
         <x:v>1.1</x:v>
@@ -9643,7 +9929,7 @@
         <x:v>https://www.prnewswire.com/news-releases/cleanspark-to-add-5-ehs-and-increase-2024-guidance-with-acquisition-of-seven-additional-bitcoin-mining-facilities-in-tennessee-302244673.html | https://www.sec.gov/Archives/edgar/data/827876/000119312525297510/clsk-20250930.htm | https://www.datacentermap.com/usa/tennessee/crossville/ | https://www.sec.gov/Archives/edgar/data/827876/000095017024105354/clsk-ex10_4.htm</x:v>
       </x:c>
       <x:c r="AF10" s="128" t="str">
-        <x:v>2026-09-04</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="AG10" s="85" t="str">
         <x:v>confirmed</x:v>
@@ -9664,7 +9950,7 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="AM10" s="85" t="str">
-        <x:v>SEC filing identifies the West Crossville property at this address; existing approximate GPS retained.</x:v>
+        <x:v>CleanSpark SEC evidence maps West Crossville Property to 268 Sparta Hwy. The separate Campbell Junction property is 5784 Plateau Rd (TNDC-002); retain two facilities and do not merge.</x:v>
       </x:c>
       <x:c r="AN10" s="85" t="str">
         <x:v>1.1</x:v>
@@ -11273,7 +11559,7 @@
         <x:v>https://baxtel.com/news/25mw-ai-data-center-planned-for-mcminnville | https://www.wsmv.com/2026/06/01/amid-plans-new-high-density-ai-data-center-campus-middle-tennessee-city-locals-push-moratorium-such-facilities/ | https://hixsondc.com/ | https://warrencountyecd.com/site/mcminnville-warren-digital-site/ | https://www.datacenterdynamics.com/en/news/25mw-ai-data-center-to-be-built-in-mcminnville-tennessee/ | https://warrencountyway.com/hixson-data-center-development-project/</x:v>
       </x:c>
       <x:c r="AF24" s="128" t="str">
-        <x:v>2026-09-04</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="AG24" s="85" t="str">
         <x:v>confirmed</x:v>
@@ -11294,7 +11580,7 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="AM24" s="85" t="str">
-        <x:v>Local reporting places the proposed site near 191 Industrial Dr; recorded as vicinity rather than exact parcel.</x:v>
+        <x:v>Hixson's current site confirms a planned 25 MW McMinnville/Warren County project but does not publish a parcel or street address. Local reporting supports only a vicinity near 191 Industrial Dr; retain this point solely as approximate_site, not as an exact parcel.</x:v>
       </x:c>
       <x:c r="AN24" s="85" t="str">
         <x:v>1.1</x:v>
@@ -12723,7 +13009,7 @@
         <x:v>Lumen Technologies Inc</x:v>
       </x:c>
       <x:c r="E37" s="23" t="str">
-        <x:v>2992 Sidco Drive</x:v>
+        <x:v>2990 Sidco Drive</x:v>
       </x:c>
       <x:c r="F37" s="17" t="str">
         <x:v>Nashville</x:v>
@@ -12779,7 +13065,7 @@
       <x:c r="Y37" s="91"/>
       <x:c r="Z37" s="35"/>
       <x:c r="AA37" s="17" t="str">
-        <x:v>peeringdb | wsmv</x:v>
+        <x:v>peeringdb | wsmv | lumen</x:v>
       </x:c>
       <x:c r="AB37" s="94" t="n">
         <x:v>2</x:v>
@@ -12788,13 +13074,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="AD37" s="23" t="str">
-        <x:v>peeringdb:311 | wsmv:nashville-list-sidco</x:v>
+        <x:v>peeringdb:311 | wsmv:nashville-list-sidco | lumen:wavelength-site-list</x:v>
       </x:c>
       <x:c r="AE37" s="23" t="str">
-        <x:v>http://www.level3.com | https://www.wsmv.com/2026/06/04/how-many-data-centers-are-there-nashville-heres-map-where-theyre-located/</x:v>
+        <x:v>http://www.level3.com | https://www.wsmv.com/2026/06/04/how-many-data-centers-are-there-nashville-heres-map-where-theyre-located/ | https://assets.lumen.com/is/content/Lumen/waves-rapid-routes-site-list</x:v>
       </x:c>
       <x:c r="AF37" s="128" t="str">
-        <x:v>2026-09-03</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="AG37" s="85" t="str">
         <x:v>confirmed</x:v>
@@ -12815,7 +13101,7 @@
         <x:v>high</x:v>
       </x:c>
       <x:c r="AM37" s="85" t="str">
-        <x:v>Address discrepancy: existing record uses 2992 Sidco Drive; independent confirmed list reports 2990 Sidco Drive. Review before parcel join.</x:v>
+        <x:v>Canonical current address is 2990 Sidco Drive from Lumen's current route list. PeeringDB's 2992 Sidco Drive is retained as an adjacent legacy-directory discrepancy; the site point remains address_or_site rather than parcel-verified.</x:v>
       </x:c>
       <x:c r="AN37" s="85" t="str">
         <x:v>1.1</x:v>
@@ -12946,10 +13232,10 @@
       <x:c r="B39" s="23" t="str">
         <x:v>Quantum Leap Data Center/ Fisk University</x:v>
       </x:c>
-      <x:c r="C39" s="23" t="str">
-        <x:v>Fisk University</x:v>
-      </x:c>
-      <x:c r="D39" s="23"/>
+      <x:c r="C39" s="23" t="str"/>
+      <x:c r="D39" s="23" t="str">
+        <x:v>Fisk University (project sponsor); operating partner not publicly identified</x:v>
+      </x:c>
       <x:c r="E39" s="23" t="str">
         <x:v>1000 17th Ave N</x:v>
       </x:c>
@@ -13028,7 +13314,7 @@
         <x:v>https://www.datacenterdynamics.com/en/news/fisk-university-looks-to-build-data-center-in-nashville-tennessee/ | https://www.fisk.edu/quantumleap/ | https://www.fisk.edu/main-featured/fisk-university-unveils-1-billion-master-plan-launching-new-era-of-innovation-and-sustainability/ | https://www.datacentermap.com/usa/tennessee/nashville/quantum-leap-data-center/ | https://www.whereorg.com/fisk-university-15250808</x:v>
       </x:c>
       <x:c r="AF39" s="128" t="str">
-        <x:v>2026-09-04</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="AG39" s="85" t="str">
         <x:v>confirmed</x:v>
@@ -13049,7 +13335,7 @@
         <x:v>high</x:v>
       </x:c>
       <x:c r="AM39" s="85" t="str">
-        <x:v>Address-level coordinate for 1000 17th Ave N; operator is Fisk University.</x:v>
+        <x:v>Fisk is the landowner and project sponsor. Fisk's August 2026 announcement describes the data-center corporate partner as yet to be determined, so no facility operator is attributed in this field.</x:v>
       </x:c>
       <x:c r="AN39" s="85" t="str">
         <x:v>1.1</x:v>
@@ -15354,10 +15640,10 @@
         <x:v>https://5c.ai/datacenters | https://5c.ai/ | https://5c.ai/news/5c-secures-more-than-usd-1-4-billion-to-power-north-americas-ai-infrastructure | https://www.assessormelvinburgess.com/propertyDetails?IR=true&amp;parcelid=073101++00119 | https://www.shelbytnhealth.com/DocumentCenter/View/7588 | https://www.datacenterdynamics.com/en/news/5c-plots-data-center-at-former-freds-site-in-memphis-tennessee/ | https://www.datacentermap.com/usa/tennessee/memphis/5cdc-memphis-mem01/ | https://baxtel.com/data-center/5cdc-memphis-tn | https://registry.deploy.report/datacenters/facilities/5c-memphis-getwell-road-tn</x:v>
       </x:c>
       <x:c r="AF59" s="123" t="str">
-        <x:v>2026-09-04</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="AG59" s="85" t="str">
-        <x:v>review</x:v>
+        <x:v>confirmed</x:v>
       </x:c>
       <x:c r="AH59" s="85" t="str">
         <x:v>identified</x:v>
@@ -15375,7 +15661,7 @@
         <x:v>medium</x:v>
       </x:c>
       <x:c r="AM59" s="85" t="str">
-        <x:v>Current DataCenterMap facility-facing address is 4280 Getwell Rd. Derived approximate-site coordinate from distances to Lumen Memphis 1 (0.38 mi), EdgeConneX Memphis (2.82 mi), and Connect Memphis (2.95 mi); residuals are effectively zero (&lt;0.001 km). Existing 4300 Getwell Rd assessor/permit evidence is preserved as related broader-site construction/property evidence, but the normalized facility address is updated to 4280 Getwell Rd.</x:v>
+        <x:v>Retain 4280 Getwell Rd as the facility-facing address supported by the current facility directory and the existing distance-derived site point. Shelby County's 4300 Getwell Rd notice is retained as related broader-site permit/property evidence, not silently substituted as the facility address.</x:v>
       </x:c>
       <x:c r="AN59" t="str">
         <x:v>1.1</x:v>
@@ -15799,7 +16085,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbad42c0300574707"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd675d4dec05a456f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36662,7 +36948,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9a37ae698d3491a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36dc408234cd43f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38704,7 +38990,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d57bebf2cb74bd4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d0c57e6acce4c93"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38827,7 +39113,9 @@
       <x:c r="O2" s="46" t="str">
         <x:v>manual_review</x:v>
       </x:c>
-      <x:c r="P2" s="43" t="str"/>
+      <x:c r="P2" s="43" t="str">
+        <x:v>xAI confirms a South Memphis Colossus facility but the generic Compute Atlas source lacks a campus identifier. Do not merge it into Colossus 1 or Colossus 2 without source-specific evidence.</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="34" hidden="0" customHeight="1">
       <x:c r="A3" s="39" t="str">
@@ -38875,12 +39163,14 @@
       <x:c r="O3" s="47" t="str">
         <x:v>manual_review</x:v>
       </x:c>
-      <x:c r="P3" s="45" t="str"/>
+      <x:c r="P3" s="45" t="str">
+        <x:v>xAI confirms a South Memphis Colossus facility but the generic Compute Atlas source lacks a campus identifier. Do not merge it into Colossus 1 or Colossus 2 without source-specific evidence.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37fb29ffda0440c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d5fb96826674ecd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -39256,7 +39546,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74aa13d3b7114f44"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfaa8b44e27e54611"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -39441,7 +39731,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4266988d073e438c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86bb6349a0ac436e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -39753,10 +40043,10 @@
         <x:v>https://www.globenewswire.com/news-release/2024/02/06/2824158/0/en/GRIID-Infrastructure-to-Add-60-MW-with-New-Bitcoin-Mining-Facility-in-Tennessee.html | https://www.prnewswire.com/news-releases/cleanspark-announces-agreement-to-acquire-griid-infrastructure-based-on-an-enterprise-value-of-155-million-and-expansion-plans-of-over-400-mw-in-tennessee-302184116.html | https://www.sec.gov/Archives/edgar/data/1830029/000119312524223759/d888816ddefm14a.htm | https://baxtel.com/data-center/cleanspark-jackson-tn | https://tpucdockets.tn.gov/archive/filings/2003/0300438ar.pdf | https://www.sec.gov/Archives/edgar/data/1830029/000119312524000728/d941597dex211.htm</x:v>
       </x:c>
       <x:c r="P5" s="123" t="str">
-        <x:v>2026-09-04</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="Q5" s="85" t="str">
-        <x:v>Jackson Energy Authority's audited filing states that Jones Creek Substation was built to serve Jackson Data, LLC located at 2342 North Parkway East and that the site would draw 60 MW of data-center load. SEC Exhibit 21.1 identifies Jackson Data LLC as a 100%-owned GRIID subsidiary; current Baxtel identifies the CleanSpark Jackson facility as operational, built 2025, on 15 acres with Jackson Energy Authority. This resolves the street address with high confidence. A defensible textual WGS84 point for 2342 North Parkway East was not found, so latitude/longitude remain blank rather than using a road-segment or nearby-business coordinate.</x:v>
+        <x:v>Public evidence supports prior GRIID/CleanSpark Jackson development and property ownership, but does not independently confirm the stated 60 MW facility is currently operating or energized. Retained as an unpromoted candidate.</x:v>
       </x:c>
       <x:c r="R5" s="85" t="str">
         <x:v>address_or_site</x:v>
@@ -39789,12 +40079,8 @@
         <x:v>TN</x:v>
       </x:c>
       <x:c r="J6"/>
-      <x:c r="K6" t="n">
-        <x:v>36.16488198</x:v>
-      </x:c>
-      <x:c r="L6" t="n">
-        <x:v>-86.78088767</x:v>
-      </x:c>
+      <x:c r="K6" t="str"/>
+      <x:c r="L6" t="str"/>
       <x:c r="M6" s="85" t="str">
         <x:v>Developer materials describe a 120 MW, 38-acre Nashville campus in development, but the exact site and county are not public.</x:v>
       </x:c>
@@ -39805,10 +40091,10 @@
         <x:v>https://atmosphere-dc.com/data-centers/nashville-tn/ | https://www.datacenterdynamics.com/en/news/atmosphere-dc-secures-investment-from-agc-equity-partners/ | https://baxtel.com/data-center/h5-data-centers-nashville-tn01 | https://baxtel.com/data-center/h5-data-centers-nashville-tn02 | https://baxtel.com/data-center/edgeconnex-nashville | https://baxtel.com/data-center/dc-blox-nashville | https://baxtel.com/data-center/lumen-nashville-2</x:v>
       </x:c>
       <x:c r="P6" s="123" t="str">
-        <x:v>2026-09-04</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="Q6" s="85" t="str">
-        <x:v>Atmosphere officially discloses only Nashville, 120 MW, and a 38-acre campus. Baxtel nearest-facility distances can be multilaterated to approximately 36.16488198, -86.78088767 with sub-0.02-mile residuals, but that point lies in the downtown carrier-hotel cluster and is physically inconsistent with a 38-acre campus. It is therefore retained only as an area_or_city / low-confidence directory market pin, NOT as the development parcel. Exclude this point from parcel/site-level spatial analyses until the actual 38-acre site is disclosed.</x:v>
+        <x:v>Atmosphere publicly discloses Nashville, 120 MW, and a 38-acre campus but no street address, county, or parcel. The previous directory-derived market pin is removed because it is physically inconsistent with a 38-acre campus. Retain as a market-level candidate only.</x:v>
       </x:c>
       <x:c r="R6" s="85" t="str">
         <x:v>area_or_city</x:v>
@@ -39816,9 +40102,7 @@
       <x:c r="S6" s="85" t="str">
         <x:v>low</x:v>
       </x:c>
-      <x:c r="T6" s="85" t="str">
-        <x:v>baxtel-derived:atmosphere-market-pin</x:v>
-      </x:c>
+      <x:c r="T6" s="85" t="str"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
@@ -40129,12 +40413,14 @@
         <x:v>Scipio Technologies NREP Listing</x:v>
       </x:c>
       <x:c r="D12" t="str">
-        <x:v>unresolved_duplicate_or_new_facility</x:v>
+        <x:v>linked_master_evidence</x:v>
       </x:c>
       <x:c r="E12" t="str">
-        <x:v>low</x:v>
-      </x:c>
-      <x:c r="F12"/>
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>1661 Murfreesboro Pike</x:v>
+      </x:c>
       <x:c r="G12" t="str">
         <x:v>Nashville</x:v>
       </x:c>
@@ -40150,7 +40436,7 @@
       <x:c r="K12"/>
       <x:c r="L12"/>
       <x:c r="M12" s="85" t="str">
-        <x:v>A current market directory lists Scipio NREP in Nashville, but the public evidence does not establish whether it is distinct from TNDC-038 at 1661 Murfreesboro Pike.</x:v>
+        <x:v>Scipio's public support address is 1661 Murfreesboro Pike, matching TNDC-038. It is retained as linked supporting evidence, not a distinct spatial candidate.</x:v>
       </x:c>
       <x:c r="N12" s="85" t="str">
         <x:v>datacentermap.com | scipiotech.com</x:v>
@@ -40159,16 +40445,16 @@
         <x:v>https://www.datacentermap.com/usa/tennessee/nashville/ | https://scipiotech.com/support/ | https://www.datacentermap.com/usa/tennessee/nashville/nexus-nrep/</x:v>
       </x:c>
       <x:c r="P12" s="123" t="str">
-        <x:v>2026-09-04</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="Q12" s="85" t="str">
-        <x:v>Explicit non-public exception: current DataCenterMap record states that the exact location is not public. Only Nashville/ZIP 37217 is public; coordinates intentionally remain blank.</x:v>
+        <x:v>Resolved as linked evidence for TNDC-038 by the shared 1661 Murfreesboro Pike address. Coordinates remain blank because this row is not a distinct site.</x:v>
       </x:c>
       <x:c r="R12" s="85" t="str">
-        <x:v>area_or_city</x:v>
+        <x:v>address_or_site</x:v>
       </x:c>
       <x:c r="S12" s="85" t="str">
-        <x:v>low</x:v>
+        <x:v>high</x:v>
       </x:c>
       <x:c r="T12" s="85"/>
     </x:row>
@@ -40217,10 +40503,10 @@
         <x:v>https://www.dataprise.com/get-in-touch/location/chattanooga/ | https://www.datacentermap.com/usa/tennessee/chattanooga/ | https://tnecd.com/wp-content/uploads/2018/10/business-services.pdf | https://www.whereorg.com/attorney-referral-service-15170587</x:v>
       </x:c>
       <x:c r="P13" s="123" t="str">
-        <x:v>2026-09-04</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="Q13" s="85" t="str">
-        <x:v>Address-level coordinate for 801 Broad St, Chattanooga.</x:v>
+        <x:v>Current directory evidence lists the Airnet/Dataprise facility at 801 Broad Street, but no primary operator page confirms current data-center operations there. Retained as a candidate pending primary operational confirmation.</x:v>
       </x:c>
       <x:c r="R13" s="85" t="str">
         <x:v>address_or_site</x:v>
@@ -40275,10 +40561,10 @@
         <x:v>https://www.datacentermap.com/usa/tennessee/nashville/nuvox-nashville/ | https://tnecd.com/wp-content/uploads/2018/10/business-services.pdf | https://www.cityfeet.com/cont/listing/940-3rd-ave-n-nashville-tn-37201/cs39837774 | https://github.com/cmusatyalab/elijah-discovery-basic/blob/master/elijah/discovery/emulation/gps</x:v>
       </x:c>
       <x:c r="P14" s="123" t="str">
-        <x:v>2026-09-04</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="Q14" s="85" t="str">
-        <x:v>DataCenterMap identifies Windstream Nashville at 940 3rd Ave North; a public geocoded GPS dataset gives 36.173667, -86.7835769 for the same address.</x:v>
+        <x:v>Current directory evidence lists the former Windstream/NuVox facility at 940 3rd Ave N. Corporate ownership naming changed after the Uniti transaction, but no primary operator page confirms current data-center operations. Retained as a candidate.</x:v>
       </x:c>
       <x:c r="R14" s="85" t="str">
         <x:v>address_or_site</x:v>
@@ -40335,10 +40621,10 @@
         <x:v>https://www.datacentermap.com/usa/tennessee/memphis/ | https://tnecd.com/wp-content/uploads/2018/10/business-services.pdf | https://www.shelbycountytn.gov/Archive/ViewFile/Item/13459 | https://promos.telarus.com/promo_docs/Q1-2011-XO-Colocation-and-DIA-Promo-Sales-Summary.pdf | https://www.whereorg.com/directv-15064353</x:v>
       </x:c>
       <x:c r="P15" s="123" t="str">
-        <x:v>2026-09-04</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="Q15" s="85" t="str">
-        <x:v>Address-level coordinate for 5127 Truse Rd, Memphis.</x:v>
+        <x:v>Current directory evidence lists a Verizon facility at 5127 Truse Rd, but no primary current facility page confirms active data-center service. Retained as a candidate.</x:v>
       </x:c>
       <x:c r="R15" s="85" t="str">
         <x:v>address_or_site</x:v>
@@ -40393,10 +40679,10 @@
         <x:v>https://tnecd.com/wp-content/uploads/2018/10/business-services.pdf | https://businessinternet.com/tennessee/memphis | https://baxtel.com/data-center/memphis | https://www.whereorg.com/conference-technologies-15266003</x:v>
       </x:c>
       <x:c r="P16" s="123" t="str">
-        <x:v>2026-09-04</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="Q16" s="85" t="str">
-        <x:v>Address-level coordinate for 5425 E Raines Rd, Memphis.</x:v>
+        <x:v>Current sources conflict: one directory labels the former tw telecom/Lumen listing inactive, while another labels it operational. Retained as a candidate with unresolved operating status.</x:v>
       </x:c>
       <x:c r="R16" s="85" t="str">
         <x:v>address_or_site</x:v>
@@ -40485,7 +40771,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11744bc9de1844c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44533988b8334e40"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Align Tennessee master feature status field
</commit_message>
<xml_diff>
--- a/TN/dataset/tennessee_public_data_centers.xlsx
+++ b/TN/dataset/tennessee_public_data_centers.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R0512b60b15d34410"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R8b59c3c957a445fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master" sheetId="3" r:id="Re6a0ad065e0e48a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw_Aligned" sheetId="4" r:id="R2b9315484dc44675"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Match_Audit" sheetId="5" r:id="R60c38f80d7ce44e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Pairs" sheetId="6" r:id="Rc7af1a06c20c4b36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded_Support" sheetId="7" r:id="R1a066b5be4d04cec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field_Map" sheetId="8" r:id="R6e67a17ff8784117"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidate_Sites" sheetId="9" r:id="Rf7cf617051f04f72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Log" sheetId="10" r:id="Ra5f3e93c3eb14f45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proposal_Readiness" sheetId="11" r:id="R8d516726ec1f4a09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Queue" sheetId="12" r:id="R94c7471464a44965"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Location_Audit" sheetId="13" r:id="Recaf2ccdc22149f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R5ac92023e7b8402a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R9e0b0a95ff024360"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master" sheetId="3" r:id="R232f2a6fcf5e4c45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw_Aligned" sheetId="4" r:id="R5bed570c70b14e06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Match_Audit" sheetId="5" r:id="R0f13595a73b44b1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Pairs" sheetId="6" r:id="R4956a203b79249cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded_Support" sheetId="7" r:id="R784c14e5afad4fe5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field_Map" sheetId="8" r:id="R92bcb7a7a9d84a4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidate_Sites" sheetId="9" r:id="Re46971f5cb76403c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Log" sheetId="10" r:id="R1008d6c561ad4825"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proposal_Readiness" sheetId="11" r:id="R5b1799a13da84214"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Queue" sheetId="12" r:id="R62431bf89c8c4840"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Location_Audit" sheetId="13" r:id="Rd205eed25ecf45e8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9256,7 +9256,7 @@
         <x:v>schema_version</x:v>
       </x:c>
       <x:c r="AO1" s="84" t="str">
-        <x:v>dataset_version</x:v>
+        <x:v>phase1_feature_status</x:v>
       </x:c>
       <x:c r="AP1" s="211" t="str">
         <x:v>nearest_neighbor_km</x:v>
@@ -9457,7 +9457,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO2" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP2" s="207" t="n">
         <x:v>3.2412571929598153</x:v>
@@ -9656,7 +9656,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO3" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP3" s="207" t="n">
         <x:v>16.5903008348662</x:v>
@@ -9857,7 +9857,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO4" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP4" s="207" t="n">
         <x:v>0.7537456534095243</x:v>
@@ -10058,7 +10058,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO5" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP5" s="207" t="n">
         <x:v>0.4108468813552908</x:v>
@@ -10257,7 +10257,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO6" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP6" s="207" t="n">
         <x:v>0.7537456534095243</x:v>
@@ -10458,7 +10458,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO7" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>city_representative_features</x:v>
       </x:c>
       <x:c r="AP7" s="207" t="n">
         <x:v>13.34786983412424</x:v>
@@ -10661,7 +10661,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO8" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP8" s="207" t="n">
         <x:v>13.34786983412424</x:v>
@@ -10864,7 +10864,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO9" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP9" s="207" t="n">
         <x:v>11.311970674520817</x:v>
@@ -11063,7 +11063,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO10" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP10" s="207" t="n">
         <x:v>16.5903008348662</x:v>
@@ -11258,7 +11258,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO11" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP11" s="207" t="n">
         <x:v>52.76647745819776</x:v>
@@ -11459,7 +11459,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO12" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP12" s="207" t="n">
         <x:v>3.2412571929598153</x:v>
@@ -11660,7 +11660,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO13" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP13" s="207" t="n">
         <x:v>3.65144110529003</x:v>
@@ -11865,7 +11865,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO14" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP14" s="207" t="n">
         <x:v>3.580764672121382</x:v>
@@ -12068,7 +12068,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO15" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP15" s="207" t="n">
         <x:v>2.3980314314913542</x:v>
@@ -12275,7 +12275,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO16" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP16" s="207" t="n">
         <x:v>2.3980314314913542</x:v>
@@ -12476,7 +12476,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO17" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP17" s="207" t="n">
         <x:v>28.99347267843897</x:v>
@@ -12677,7 +12677,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO18" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP18" s="207" t="n">
         <x:v>7.584785746838801</x:v>
@@ -12876,7 +12876,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO19" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP19" s="207" t="n">
         <x:v>0.992513351398504</x:v>
@@ -13077,7 +13077,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO20" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP20" s="207" t="n">
         <x:v>4.917109437996493</x:v>
@@ -13272,7 +13272,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO21" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP21" s="207" t="n">
         <x:v>57.045255277578455</x:v>
@@ -13469,7 +13469,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO22" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP22" s="207" t="n">
         <x:v>43.6773958414442</x:v>
@@ -13664,7 +13664,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO23" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP23" s="207" t="n">
         <x:v>27.74221155274318</x:v>
@@ -13869,7 +13869,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO24" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP24" s="207" t="n">
         <x:v>7.55864423304588</x:v>
@@ -14068,7 +14068,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO25" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP25" s="207" t="n">
         <x:v>7.55864423304588</x:v>
@@ -14269,7 +14269,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO26" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP26" s="207" t="n">
         <x:v>6.5393152771957945</x:v>
@@ -14468,7 +14468,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO27" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP27" s="207" t="n">
         <x:v>0.3454071544348475</x:v>
@@ -14673,7 +14673,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO28" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP28" s="207" t="n">
         <x:v>9.26082548446652</x:v>
@@ -14872,7 +14872,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO29" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP29" s="207" t="n">
         <x:v>0.6115269873530994</x:v>
@@ -15073,7 +15073,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO30" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP30" s="207" t="n">
         <x:v>12.992330991063133</x:v>
@@ -15278,7 +15278,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO31" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP31" s="207" t="n">
         <x:v>9.853330615022765</x:v>
@@ -15481,7 +15481,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO32" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP32" s="207" t="n">
         <x:v>1.5634296886992427</x:v>
@@ -15680,7 +15680,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO33" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP33" s="207" t="n">
         <x:v>1.976314023135052</x:v>
@@ -15883,7 +15883,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO34" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP34" s="207" t="n">
         <x:v>0.2086854803185778</x:v>
@@ -16084,7 +16084,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO35" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP35" s="207" t="n">
         <x:v>0.2086854803185778</x:v>
@@ -16283,7 +16283,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO36" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP36" s="207" t="n">
         <x:v>2.3989227738591374</x:v>
@@ -16482,7 +16482,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO37" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP37" s="207" t="n">
         <x:v>1.5634296886992427</x:v>
@@ -16681,7 +16681,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO38" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP38" s="207" t="n">
         <x:v>5.053066150501399</x:v>
@@ -16884,7 +16884,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO39" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP39" s="207" t="n">
         <x:v>1.735944713176277</x:v>
@@ -17085,7 +17085,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO40" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP40" s="207" t="n">
         <x:v>10.252603292630416</x:v>
@@ -17284,7 +17284,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO41" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP41" s="207" t="n">
         <x:v>0.5416832532175047</x:v>
@@ -17483,7 +17483,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO42" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP42" s="207" t="n">
         <x:v>0.919336050690768</x:v>
@@ -17684,7 +17684,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO43" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP43" s="207" t="n">
         <x:v>27.74221155274318</x:v>
@@ -17879,7 +17879,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO44" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP44" s="207" t="n">
         <x:v>7.65235803152038</x:v>
@@ -18078,7 +18078,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO45" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP45" s="207" t="n">
         <x:v>7.65235803152038</x:v>
@@ -18277,7 +18277,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO46" s="85" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP46" s="207" t="n">
         <x:v>4.917109437996493</x:v>
@@ -18478,7 +18478,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO47" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP47" s="207" t="n">
         <x:v>0.992513351398504</x:v>
@@ -18677,7 +18677,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO48" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP48" s="207" t="n">
         <x:v>1.4454623860169304</x:v>
@@ -18876,7 +18876,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO49" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP49" s="207" t="n">
         <x:v>1.4454623860169304</x:v>
@@ -19075,7 +19075,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO50" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP50" s="207" t="n">
         <x:v>4.365935265331043</x:v>
@@ -19278,7 +19278,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO51" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP51" s="207" t="n">
         <x:v>10.771741932562746</x:v>
@@ -19481,7 +19481,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO52" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP52" s="207" t="n">
         <x:v>17.477420413451394</x:v>
@@ -19682,7 +19682,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO53" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP53" s="207" t="n">
         <x:v>7.201622189296421</x:v>
@@ -19883,7 +19883,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO54" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP54" s="207" t="n">
         <x:v>1.976314023135052</x:v>
@@ -20084,7 +20084,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO55" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP55" s="207" t="n">
         <x:v>1.510841476707156</x:v>
@@ -20287,7 +20287,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO56" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP56" s="207" t="n">
         <x:v>1.510841476707156</x:v>
@@ -20486,7 +20486,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO57" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP57" s="207" t="n">
         <x:v>0.536086088636087</x:v>
@@ -20687,7 +20687,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO58" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP58" s="207" t="n">
         <x:v>0.3454071544348475</x:v>
@@ -20890,7 +20890,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO59" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP59" s="207" t="n">
         <x:v>0.6115269873530994</x:v>
@@ -21093,7 +21093,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO60" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP60" s="207" t="n">
         <x:v>6.183699762877351</x:v>
@@ -21294,7 +21294,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO61" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP61" s="207" t="n">
         <x:v>23.739097663615286</x:v>
@@ -21499,7 +21499,7 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="AO62" t="str">
-        <x:v>2026-09-03-deduplicated</x:v>
+        <x:v>direct_site_features</x:v>
       </x:c>
       <x:c r="AP62" s="207" t="n">
         <x:v>37.94409711967336</x:v>
@@ -21644,7 +21644,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36774806f8c84305"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re95a139c1903423d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -42507,7 +42507,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa50700318684d03"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8dc61433c7f54361"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -44549,7 +44549,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R425b4b3ecadb40c0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13159f9452744b72"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -44729,7 +44729,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c237ebd7bfa4ad6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd5a0bfeaa8e4763"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -45105,7 +45105,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd208a7c1e3cd49e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e4a0a7040164ae7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -45290,7 +45290,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1cea2fdd68ae42bd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5364e476327c4262"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -47860,7 +47860,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf83bec226d04b5c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R666dc95281814e48"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Synchronize Tennessee master table headers
</commit_message>
<xml_diff>
--- a/TN/dataset/tennessee_public_data_centers.xlsx
+++ b/TN/dataset/tennessee_public_data_centers.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R5ac92023e7b8402a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R9e0b0a95ff024360"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master" sheetId="3" r:id="R232f2a6fcf5e4c45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw_Aligned" sheetId="4" r:id="R5bed570c70b14e06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Match_Audit" sheetId="5" r:id="R0f13595a73b44b1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Pairs" sheetId="6" r:id="R4956a203b79249cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded_Support" sheetId="7" r:id="R784c14e5afad4fe5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field_Map" sheetId="8" r:id="R92bcb7a7a9d84a4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidate_Sites" sheetId="9" r:id="Re46971f5cb76403c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Log" sheetId="10" r:id="R1008d6c561ad4825"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proposal_Readiness" sheetId="11" r:id="R5b1799a13da84214"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Queue" sheetId="12" r:id="R62431bf89c8c4840"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Location_Audit" sheetId="13" r:id="Rd205eed25ecf45e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rf732e16e46704712"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R5cb4edc09a244fb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master" sheetId="3" r:id="R5e31e578ccb04039"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw_Aligned" sheetId="4" r:id="R1c0487e55c8549e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Match_Audit" sheetId="5" r:id="Ree74a0fb191842f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Pairs" sheetId="6" r:id="Raeaf0a7341894ac8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded_Support" sheetId="7" r:id="Racbb828dc1f7499b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field_Map" sheetId="8" r:id="Rb8265469b1914b08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidate_Sites" sheetId="9" r:id="R0e6bc051f87f481e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Log" sheetId="10" r:id="Rb9783db99aa04d33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proposal_Readiness" sheetId="11" r:id="R8a4ad03fb1cd47f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Queue" sheetId="12" r:id="Rbd0d7233d545407f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Location_Audit" sheetId="13" r:id="R3e14e02811584a18"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1007,7 +1007,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="MasterTable" displayName="MasterTable" ref="A1:BQ62" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="MasterTable" displayName="MasterTable" ref="A1:BQ62" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="69">
     <x:tableColumn id="1" name="facility_id"/>
     <x:tableColumn id="2" name="facility_name"/>
@@ -1049,35 +1049,35 @@
     <x:tableColumn id="38" name="source_confidence_class"/>
     <x:tableColumn id="39" name="verification_note"/>
     <x:tableColumn id="40" name="schema_version"/>
-    <x:tableColumn id="41" name="dataset_version"/>
-    <x:tableColumn id="42" name="dataset_version"/>
-    <x:tableColumn id="43" name="dataset_version"/>
-    <x:tableColumn id="44" name="dataset_version"/>
-    <x:tableColumn id="45" name="dataset_version"/>
-    <x:tableColumn id="46" name="dataset_version"/>
-    <x:tableColumn id="47" name="dataset_version"/>
-    <x:tableColumn id="48" name="dataset_version"/>
-    <x:tableColumn id="49" name="dataset_version"/>
-    <x:tableColumn id="50" name="dataset_version"/>
-    <x:tableColumn id="51" name="dataset_version"/>
-    <x:tableColumn id="52" name="dataset_version"/>
-    <x:tableColumn id="53" name="dataset_version"/>
-    <x:tableColumn id="54" name="dataset_version"/>
-    <x:tableColumn id="55" name="dataset_version"/>
-    <x:tableColumn id="56" name="dataset_version"/>
-    <x:tableColumn id="57" name="dataset_version"/>
-    <x:tableColumn id="58" name="dataset_version"/>
-    <x:tableColumn id="59" name="dataset_version"/>
-    <x:tableColumn id="60" name="dataset_version"/>
-    <x:tableColumn id="61" name="dataset_version"/>
-    <x:tableColumn id="62" name="dataset_version"/>
-    <x:tableColumn id="63" name="dataset_version"/>
-    <x:tableColumn id="64" name="dataset_version"/>
-    <x:tableColumn id="65" name="dataset_version"/>
-    <x:tableColumn id="66" name="dataset_version"/>
-    <x:tableColumn id="67" name="dataset_version"/>
-    <x:tableColumn id="68" name="dataset_version"/>
-    <x:tableColumn id="69" name="dataset_version"/>
+    <x:tableColumn id="41" name="phase1_feature_status"/>
+    <x:tableColumn id="42" name="nearest_neighbor_km"/>
+    <x:tableColumn id="43" name="cluster"/>
+    <x:tableColumn id="44" name="dist_transmission_any_km"/>
+    <x:tableColumn id="45" name="dist_transmission_100kv_km"/>
+    <x:tableColumn id="46" name="dist_transmission_230kv_km"/>
+    <x:tableColumn id="47" name="max_voltage_within_25km_kv"/>
+    <x:tableColumn id="48" name="transmission_owner_count_25km"/>
+    <x:tableColumn id="49" name="dist_major_road_km"/>
+    <x:tableColumn id="50" name="dist_interstate_km"/>
+    <x:tableColumn id="51" name="dist_surface_water_flowline_km"/>
+    <x:tableColumn id="52" name="named_flowlines_within_25km"/>
+    <x:tableColumn id="53" name="county_geoid"/>
+    <x:tableColumn id="54" name="county_name"/>
+    <x:tableColumn id="55" name="degree_institutions_50km"/>
+    <x:tableColumn id="56" name="cip11_completions_50km"/>
+    <x:tableColumn id="57" name="cip14_completions_50km"/>
+    <x:tableColumn id="58" name="degree_institutions_100km"/>
+    <x:tableColumn id="59" name="cip11_completions_100km"/>
+    <x:tableColumn id="60" name="cip14_completions_100km"/>
+    <x:tableColumn id="61" name="county_total_employment"/>
+    <x:tableColumn id="62" name="county_total_establishments"/>
+    <x:tableColumn id="63" name="county_total_employment_flag"/>
+    <x:tableColumn id="64" name="information_sector_employment"/>
+    <x:tableColumn id="65" name="information_sector_establishments"/>
+    <x:tableColumn id="66" name="information_sector_employment_flag"/>
+    <x:tableColumn id="67" name="professional_scientific_employment"/>
+    <x:tableColumn id="68" name="professional_scientific_establishments"/>
+    <x:tableColumn id="69" name="professional_scientific_employment_flag"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -21644,7 +21644,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re95a139c1903423d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc26811007a54dd5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -42507,7 +42507,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8dc61433c7f54361"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3e8f7d618ce4d76"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -44549,7 +44549,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13159f9452744b72"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d25c43b0a85430e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -44729,7 +44729,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd5a0bfeaa8e4763"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a11a23e9dcc4dac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -45105,7 +45105,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e4a0a7040164ae7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc738802101c448b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -45290,7 +45290,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5364e476327c4262"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33cb1e09435e4ce0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -47860,7 +47860,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R666dc95281814e48"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea7a800858b640b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh Tennessee model artifacts and English research materials
</commit_message>
<xml_diff>
--- a/TN/dataset/tennessee_public_data_centers.xlsx
+++ b/TN/dataset/tennessee_public_data_centers.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rf732e16e46704712"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R5cb4edc09a244fb2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master" sheetId="3" r:id="R5e31e578ccb04039"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw_Aligned" sheetId="4" r:id="R1c0487e55c8549e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Match_Audit" sheetId="5" r:id="Ree74a0fb191842f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Pairs" sheetId="6" r:id="Raeaf0a7341894ac8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded_Support" sheetId="7" r:id="Racbb828dc1f7499b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field_Map" sheetId="8" r:id="Rb8265469b1914b08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidate_Sites" sheetId="9" r:id="R0e6bc051f87f481e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Log" sheetId="10" r:id="Rb9783db99aa04d33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proposal_Readiness" sheetId="11" r:id="R8a4ad03fb1cd47f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Queue" sheetId="12" r:id="Rbd0d7233d545407f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Location_Audit" sheetId="13" r:id="R3e14e02811584a18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R22ced22afa04408b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R84377b1ec7ca48ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master" sheetId="3" r:id="Rc02ad912dec3421f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw_Aligned" sheetId="4" r:id="R22d80092e3f0456b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Match_Audit" sheetId="5" r:id="Raadf8416d1374666"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Pairs" sheetId="6" r:id="R3db9656abf144276"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded_Support" sheetId="7" r:id="R34b329f8b75147bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field_Map" sheetId="8" r:id="R070a6e16bf3c4c74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidate_Sites" sheetId="9" r:id="R9e1a0d21524c415f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Log" sheetId="10" r:id="R0b1481f32fd14c3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proposal_Readiness" sheetId="11" r:id="R0a937ec845a1433f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Queue" sheetId="12" r:id="Rb9041d75443f4a91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Location_Audit" sheetId="13" r:id="R6dbcda47173e43bb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -108,7 +108,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="23">
+  <x:fills count="24">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -213,6 +213,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF153B5B"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -379,7 +384,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="230">
+  <x:cellXfs count="234">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -982,6 +987,14 @@
     <x:xf numFmtId="204" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1713,6 +1726,60 @@
       </x:c>
       <x:c r="D22" s="85"/>
     </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="233" t="str">
+        <x:v>Phase 2 spatial domain and provenance</x:v>
+      </x:c>
+      <x:c r="B23" s="233" t="str"/>
+      <x:c r="C23" s="233" t="str"/>
+      <x:c r="D23" s="233" t="str"/>
+      <x:c r="E23" s="233" t="str"/>
+      <x:c r="F23" s="233" t="str"/>
+      <x:c r="G23" s="233" t="str"/>
+      <x:c r="H23" s="233" t="str"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>Method</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>5 km equal-area Tennessee grid; D1 removes NHD open water, PAD-US GAP 1–2 permanent protections, DFIRM explicit FLOODWAY polygons, and mean 3DEP slope &gt;=15°</x:v>
+      </x:c>
+      <x:c r="C24" t="str"/>
+      <x:c r="D24" t="str"/>
+      <x:c r="E24" t="str"/>
+      <x:c r="F24" t="str"/>
+      <x:c r="G24" t="str"/>
+      <x:c r="H24" t="str"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="str">
+        <x:v>Sources</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>USGS 3DEP ImageServer; USGS PAD-US; Tennessee DFIRM; USGS NHD; accessed 2026-09-11</x:v>
+      </x:c>
+      <x:c r="C25" t="str"/>
+      <x:c r="D25" t="str"/>
+      <x:c r="E25" t="str"/>
+      <x:c r="F25" t="str"/>
+      <x:c r="G25" t="str"/>
+      <x:c r="H25" t="str"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="str">
+        <x:v>Model copy</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>model/phase 2/dataset/phase2_model_dataset.xlsx is the only model data copy; Master and Candidate_Sites are authoritative.</x:v>
+      </x:c>
+      <x:c r="C26" t="str"/>
+      <x:c r="D26" t="str"/>
+      <x:c r="E26" t="str"/>
+      <x:c r="F26" t="str"/>
+      <x:c r="G26" t="str"/>
+      <x:c r="H26" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
@@ -9342,6 +9409,54 @@
       <x:c r="BQ1" s="212" t="str">
         <x:v>professional_scientific_employment_flag</x:v>
       </x:c>
+      <x:c r="BR1" s="233" t="str">
+        <x:v>phase2_site_id</x:v>
+      </x:c>
+      <x:c r="BS1" s="233" t="str">
+        <x:v>phase2_domain_cell_id</x:v>
+      </x:c>
+      <x:c r="BT1" s="233" t="str">
+        <x:v>phase2_d1_feasible</x:v>
+      </x:c>
+      <x:c r="BU1" s="233" t="str">
+        <x:v>phase2_d1_exclusion_reason</x:v>
+      </x:c>
+      <x:c r="BV1" s="233" t="str">
+        <x:v>phase2_open_water_flag</x:v>
+      </x:c>
+      <x:c r="BW1" s="233" t="str">
+        <x:v>phase2_protected_land_flag</x:v>
+      </x:c>
+      <x:c r="BX1" s="233" t="str">
+        <x:v>phase2_regulatory_floodway_flag</x:v>
+      </x:c>
+      <x:c r="BY1" s="233" t="str">
+        <x:v>phase2_mean_slope_deg</x:v>
+      </x:c>
+      <x:c r="BZ1" s="233" t="str">
+        <x:v>phase2_urban_context</x:v>
+      </x:c>
+      <x:c r="CA1" s="233" t="str">
+        <x:v>phase2_developed_context</x:v>
+      </x:c>
+      <x:c r="CB1" s="233" t="str">
+        <x:v>phase2_grand_region</x:v>
+      </x:c>
+      <x:c r="CC1" s="233" t="str">
+        <x:v>phase2_primary_weight</x:v>
+      </x:c>
+      <x:c r="CD1" s="233" t="str">
+        <x:v>phase2_weighted_weight</x:v>
+      </x:c>
+      <x:c r="CE1" s="233" t="str">
+        <x:v>phase2_strict_weight</x:v>
+      </x:c>
+      <x:c r="CF1" s="233" t="str">
+        <x:v>phase2_feature_status</x:v>
+      </x:c>
+      <x:c r="CG1" s="233" t="str">
+        <x:v>phase2_evidence_urls</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="30" hidden="0" customHeight="1">
       <x:c r="A2" s="13" t="str">
@@ -9543,6 +9658,54 @@
       <x:c r="BQ2" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR2" t="str">
+        <x:v>TNDC-001</x:v>
+      </x:c>
+      <x:c r="BS2" t="str">
+        <x:v>TN5K-1967</x:v>
+      </x:c>
+      <x:c r="BT2" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU2" t="str">
+        <x:v>regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV2" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BW2" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX2" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY2" t="str">
+        <x:v>0.8639828794532352</x:v>
+      </x:c>
+      <x:c r="BZ2" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA2" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB2" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="CC2" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD2" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE2" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF2" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG2" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="30" hidden="0" customHeight="1">
       <x:c r="A3" s="16" t="str">
@@ -9742,6 +9905,54 @@
       <x:c r="BQ3" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR3" t="str">
+        <x:v>TNDC-002</x:v>
+      </x:c>
+      <x:c r="BS3" t="str">
+        <x:v>TN5K-3013</x:v>
+      </x:c>
+      <x:c r="BT3" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU3" t="str">
+        <x:v>open_water</x:v>
+      </x:c>
+      <x:c r="BV3" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW3" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX3" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BY3" t="str">
+        <x:v>1.1295460379785962</x:v>
+      </x:c>
+      <x:c r="BZ3" t="str">
+        <x:v>nonmetro</x:v>
+      </x:c>
+      <x:c r="CA3" t="str">
+        <x:v>nonmetro_proxy</x:v>
+      </x:c>
+      <x:c r="CB3" t="str">
+        <x:v>east</x:v>
+      </x:c>
+      <x:c r="CC3" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD3" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE3" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF3" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG3" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="30" hidden="0" customHeight="1">
       <x:c r="A4" s="16" t="str">
@@ -9943,6 +10154,54 @@
       <x:c r="BQ4" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR4" t="str">
+        <x:v>TNDC-003</x:v>
+      </x:c>
+      <x:c r="BS4" t="str">
+        <x:v>TN5K-3027</x:v>
+      </x:c>
+      <x:c r="BT4" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU4" t="str">
+        <x:v>regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV4" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BW4" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX4" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY4" t="str">
+        <x:v>1.355089758005407</x:v>
+      </x:c>
+      <x:c r="BZ4" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA4" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB4" t="str">
+        <x:v>east</x:v>
+      </x:c>
+      <x:c r="CC4" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD4" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE4" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF4" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG4" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="30" hidden="0" customHeight="1">
       <x:c r="A5" s="16" t="str">
@@ -10144,6 +10403,54 @@
       <x:c r="BQ5" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR5" t="str">
+        <x:v>TNDC-004</x:v>
+      </x:c>
+      <x:c r="BS5" t="str">
+        <x:v>TN5K-3028</x:v>
+      </x:c>
+      <x:c r="BT5" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU5" t="str">
+        <x:v>protected_land;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV5" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BW5" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BX5" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY5" t="str">
+        <x:v>1.0866958482397928</x:v>
+      </x:c>
+      <x:c r="BZ5" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA5" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB5" t="str">
+        <x:v>east</x:v>
+      </x:c>
+      <x:c r="CC5" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD5" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE5" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF5" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG5" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="30" hidden="0" customHeight="1">
       <x:c r="A6" s="16" t="str">
@@ -10343,6 +10650,54 @@
       <x:c r="BQ6" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR6" t="str">
+        <x:v>TNDC-005</x:v>
+      </x:c>
+      <x:c r="BS6" t="str">
+        <x:v>TN5K-3028</x:v>
+      </x:c>
+      <x:c r="BT6" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU6" t="str">
+        <x:v>protected_land;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV6" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BW6" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BX6" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY6" t="str">
+        <x:v>1.0866958482397928</x:v>
+      </x:c>
+      <x:c r="BZ6" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA6" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB6" t="str">
+        <x:v>east</x:v>
+      </x:c>
+      <x:c r="CC6" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD6" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE6" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF6" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG6" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="30" hidden="0" customHeight="1">
       <x:c r="A7" s="16" t="str">
@@ -10543,6 +10898,54 @@
       </x:c>
       <x:c r="BQ7" s="209" t="str">
         <x:v>G</x:v>
+      </x:c>
+      <x:c r="BR7" t="str">
+        <x:v>TNDC-006</x:v>
+      </x:c>
+      <x:c r="BS7" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BT7" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BU7" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BV7" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BW7" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BX7" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BY7" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BZ7" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="CA7" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="CB7" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="CC7" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="CD7" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="CE7" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="CF7" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="CG7" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="30" hidden="0" customHeight="1">
@@ -10747,6 +11150,54 @@
       <x:c r="BQ8" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR8" t="str">
+        <x:v>TNDC-007</x:v>
+      </x:c>
+      <x:c r="BS8" t="str">
+        <x:v>TN5K-1608</x:v>
+      </x:c>
+      <x:c r="BT8" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU8" t="str">
+        <x:v>open_water</x:v>
+      </x:c>
+      <x:c r="BV8" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW8" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX8" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BY8" t="str">
+        <x:v>0.43263573985960746</x:v>
+      </x:c>
+      <x:c r="BZ8" t="str">
+        <x:v>nonmetro</x:v>
+      </x:c>
+      <x:c r="CA8" t="str">
+        <x:v>nonmetro_proxy</x:v>
+      </x:c>
+      <x:c r="CB8" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="CC8" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD8" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE8" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF8" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG8" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="30" hidden="0" customHeight="1">
       <x:c r="A9" s="16" t="str">
@@ -10949,6 +11400,54 @@
       </x:c>
       <x:c r="BQ9" s="209" t="str">
         <x:v>G</x:v>
+      </x:c>
+      <x:c r="BR9" t="str">
+        <x:v>TNDC-008</x:v>
+      </x:c>
+      <x:c r="BS9" t="str">
+        <x:v>TN5K-0168</x:v>
+      </x:c>
+      <x:c r="BT9" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU9" t="str">
+        <x:v>open_water;protected_land;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV9" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW9" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BX9" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY9" t="str">
+        <x:v>0.3893086314201355</x:v>
+      </x:c>
+      <x:c r="BZ9" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA9" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB9" t="str">
+        <x:v>west</x:v>
+      </x:c>
+      <x:c r="CC9" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD9" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE9" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF9" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG9" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="30" hidden="0" customHeight="1">
@@ -11149,6 +11648,54 @@
       <x:c r="BQ10" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR10" t="str">
+        <x:v>TNDC-009</x:v>
+      </x:c>
+      <x:c r="BS10" t="str">
+        <x:v>TN5K-3122</x:v>
+      </x:c>
+      <x:c r="BT10" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU10" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV10" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW10" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX10" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY10" t="str">
+        <x:v>0.5407882365915511</x:v>
+      </x:c>
+      <x:c r="BZ10" t="str">
+        <x:v>nonmetro</x:v>
+      </x:c>
+      <x:c r="CA10" t="str">
+        <x:v>nonmetro_proxy</x:v>
+      </x:c>
+      <x:c r="CB10" t="str">
+        <x:v>east</x:v>
+      </x:c>
+      <x:c r="CC10" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD10" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE10" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF10" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG10" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="30" hidden="0" customHeight="1">
       <x:c r="A11" s="16" t="str">
@@ -11344,6 +11891,54 @@
       <x:c r="BQ11" s="209" t="str">
         <x:v>NO_PUBLISHED_ROW</x:v>
       </x:c>
+      <x:c r="BR11" t="str">
+        <x:v>TNDC-010</x:v>
+      </x:c>
+      <x:c r="BS11" t="str">
+        <x:v>TN5K-3336</x:v>
+      </x:c>
+      <x:c r="BT11" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU11" t="str">
+        <x:v>regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV11" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BW11" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX11" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY11" t="str">
+        <x:v>1.7219926979806688</x:v>
+      </x:c>
+      <x:c r="BZ11" t="str">
+        <x:v>nonmetro</x:v>
+      </x:c>
+      <x:c r="CA11" t="str">
+        <x:v>nonmetro_proxy</x:v>
+      </x:c>
+      <x:c r="CB11" t="str">
+        <x:v>east</x:v>
+      </x:c>
+      <x:c r="CC11" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD11" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE11" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF11" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG11" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="30" hidden="0" customHeight="1">
       <x:c r="A12" s="16" t="str">
@@ -11545,6 +12140,54 @@
       <x:c r="BQ12" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR12" t="str">
+        <x:v>TNDC-011</x:v>
+      </x:c>
+      <x:c r="BS12" t="str">
+        <x:v>TN5K-1928</x:v>
+      </x:c>
+      <x:c r="BT12" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU12" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV12" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW12" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX12" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY12" t="str">
+        <x:v>1.095819354057312</x:v>
+      </x:c>
+      <x:c r="BZ12" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA12" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB12" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="CC12" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD12" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE12" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF12" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG12" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="30" hidden="0" customHeight="1">
       <x:c r="A13" s="16" t="str">
@@ -11746,6 +12389,54 @@
       <x:c r="BQ13" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR13" t="str">
+        <x:v>TNDC-012</x:v>
+      </x:c>
+      <x:c r="BS13" t="str">
+        <x:v>TN5K-1965</x:v>
+      </x:c>
+      <x:c r="BT13" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU13" t="str">
+        <x:v>regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV13" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BW13" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX13" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY13" t="str">
+        <x:v>0.6818343566523658</x:v>
+      </x:c>
+      <x:c r="BZ13" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA13" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB13" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="CC13" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD13" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE13" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF13" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG13" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="30" hidden="0" customHeight="1">
       <x:c r="A14" s="16" t="str">
@@ -11950,6 +12641,54 @@
       </x:c>
       <x:c r="BQ14" s="209" t="str">
         <x:v>G</x:v>
+      </x:c>
+      <x:c r="BR14" t="str">
+        <x:v>TNDC-013</x:v>
+      </x:c>
+      <x:c r="BS14" t="str">
+        <x:v>TN5K-1927</x:v>
+      </x:c>
+      <x:c r="BT14" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU14" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV14" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW14" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX14" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY14" t="str">
+        <x:v>0.6528879470295377</x:v>
+      </x:c>
+      <x:c r="BZ14" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA14" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB14" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="CC14" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD14" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE14" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF14" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG14" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="30" hidden="0" customHeight="1">
@@ -12154,6 +12893,54 @@
       <x:c r="BQ15" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR15" t="str">
+        <x:v>TNDC-014</x:v>
+      </x:c>
+      <x:c r="BS15" t="str">
+        <x:v>TN5K-2199</x:v>
+      </x:c>
+      <x:c r="BT15" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU15" t="str">
+        <x:v>regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV15" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BW15" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX15" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY15" t="str">
+        <x:v>0.827479319439994</x:v>
+      </x:c>
+      <x:c r="BZ15" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA15" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB15" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="CC15" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD15" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE15" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF15" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG15" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="30" hidden="0" customHeight="1">
       <x:c r="A16" s="16" t="str">
@@ -12360,6 +13147,54 @@
       </x:c>
       <x:c r="BQ16" s="209" t="str">
         <x:v>G</x:v>
+      </x:c>
+      <x:c r="BR16" t="str">
+        <x:v>TNDC-015</x:v>
+      </x:c>
+      <x:c r="BS16" t="str">
+        <x:v>TN5K-2199</x:v>
+      </x:c>
+      <x:c r="BT16" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU16" t="str">
+        <x:v>regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV16" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BW16" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX16" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY16" t="str">
+        <x:v>0.827479319439994</x:v>
+      </x:c>
+      <x:c r="BZ16" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA16" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB16" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="CC16" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD16" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE16" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF16" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG16" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="30" hidden="0" customHeight="1">
@@ -12562,6 +13397,54 @@
       <x:c r="BQ17" s="209" t="str">
         <x:v>H</x:v>
       </x:c>
+      <x:c r="BR17" t="str">
+        <x:v>TNDC-016</x:v>
+      </x:c>
+      <x:c r="BS17" t="str">
+        <x:v>TN5K-3658</x:v>
+      </x:c>
+      <x:c r="BT17" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU17" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV17" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW17" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX17" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY17" t="str">
+        <x:v>4.209807568126255</x:v>
+      </x:c>
+      <x:c r="BZ17" t="str">
+        <x:v>nonmetro</x:v>
+      </x:c>
+      <x:c r="CA17" t="str">
+        <x:v>nonmetro_proxy</x:v>
+      </x:c>
+      <x:c r="CB17" t="str">
+        <x:v>east</x:v>
+      </x:c>
+      <x:c r="CC17" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD17" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE17" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF17" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG17" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="30" hidden="0" customHeight="1">
       <x:c r="A18" s="16" t="str">
@@ -12762,6 +13645,54 @@
       </x:c>
       <x:c r="BQ18" s="209" t="str">
         <x:v>G</x:v>
+      </x:c>
+      <x:c r="BR18" t="str">
+        <x:v>TNDC-017</x:v>
+      </x:c>
+      <x:c r="BS18" t="str">
+        <x:v>TN5K-3861</x:v>
+      </x:c>
+      <x:c r="BT18" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU18" t="str">
+        <x:v>protected_land;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV18" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BW18" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BX18" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY18" t="str">
+        <x:v>1.1271323694123163</x:v>
+      </x:c>
+      <x:c r="BZ18" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA18" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB18" t="str">
+        <x:v>east</x:v>
+      </x:c>
+      <x:c r="CC18" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD18" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE18" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF18" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG18" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="30" hidden="0" customHeight="1">
@@ -12962,6 +13893,54 @@
       <x:c r="BQ19" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR19" t="str">
+        <x:v>TNDC-018</x:v>
+      </x:c>
+      <x:c r="BS19" t="str">
+        <x:v>TN5K-3835</x:v>
+      </x:c>
+      <x:c r="BT19" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU19" t="str">
+        <x:v>protected_land;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV19" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BW19" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BX19" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY19" t="str">
+        <x:v>1.6440967056486342</x:v>
+      </x:c>
+      <x:c r="BZ19" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA19" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB19" t="str">
+        <x:v>east</x:v>
+      </x:c>
+      <x:c r="CC19" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD19" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE19" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF19" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG19" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="30" hidden="0" customHeight="1">
       <x:c r="A20" s="16" t="str">
@@ -13162,6 +14141,54 @@
       </x:c>
       <x:c r="BQ20" s="209" t="str">
         <x:v>H</x:v>
+      </x:c>
+      <x:c r="BR20" t="str">
+        <x:v>TNDC-019</x:v>
+      </x:c>
+      <x:c r="BS20" t="str">
+        <x:v>TN5K-3641</x:v>
+      </x:c>
+      <x:c r="BT20" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU20" t="str">
+        <x:v>regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV20" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BW20" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX20" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY20" t="str">
+        <x:v>1.2509022156397502</x:v>
+      </x:c>
+      <x:c r="BZ20" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA20" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB20" t="str">
+        <x:v>east</x:v>
+      </x:c>
+      <x:c r="CC20" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD20" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE20" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF20" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG20" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="30" hidden="0" customHeight="1">
@@ -13358,6 +14385,54 @@
       <x:c r="BQ21" s="209" t="str">
         <x:v>H</x:v>
       </x:c>
+      <x:c r="BR21" t="str">
+        <x:v>TNDC-020</x:v>
+      </x:c>
+      <x:c r="BS21" t="str">
+        <x:v>TN5K-4312</x:v>
+      </x:c>
+      <x:c r="BT21" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU21" t="str">
+        <x:v>protected_land</x:v>
+      </x:c>
+      <x:c r="BV21" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BW21" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BX21" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BY21" t="str">
+        <x:v>0.6789027286900414</x:v>
+      </x:c>
+      <x:c r="BZ21" t="str">
+        <x:v>nonmetro</x:v>
+      </x:c>
+      <x:c r="CA21" t="str">
+        <x:v>nonmetro_proxy</x:v>
+      </x:c>
+      <x:c r="CB21" t="str">
+        <x:v>east</x:v>
+      </x:c>
+      <x:c r="CC21" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD21" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE21" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF21" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG21" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="30" hidden="0" customHeight="1">
       <x:c r="A22" s="16" t="str">
@@ -13554,6 +14629,54 @@
       </x:c>
       <x:c r="BQ22" s="209" t="str">
         <x:v>H</x:v>
+      </x:c>
+      <x:c r="BR22" t="str">
+        <x:v>TNDC-021</x:v>
+      </x:c>
+      <x:c r="BS22" t="str">
+        <x:v>TN5K-2477</x:v>
+      </x:c>
+      <x:c r="BT22" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU22" t="str">
+        <x:v>open_water</x:v>
+      </x:c>
+      <x:c r="BV22" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW22" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX22" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BY22" t="str">
+        <x:v>0.2577753828631507</x:v>
+      </x:c>
+      <x:c r="BZ22" t="str">
+        <x:v>nonmetro</x:v>
+      </x:c>
+      <x:c r="CA22" t="str">
+        <x:v>nonmetro_proxy</x:v>
+      </x:c>
+      <x:c r="CB22" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="CC22" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD22" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE22" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF22" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG22" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="30" hidden="0" customHeight="1">
@@ -13750,6 +14873,54 @@
       <x:c r="BQ23" s="209" t="str">
         <x:v>J</x:v>
       </x:c>
+      <x:c r="BR23" t="str">
+        <x:v>TNDC-022</x:v>
+      </x:c>
+      <x:c r="BS23" t="str">
+        <x:v>TN5K-3868</x:v>
+      </x:c>
+      <x:c r="BT23" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU23" t="str">
+        <x:v>open_water</x:v>
+      </x:c>
+      <x:c r="BV23" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW23" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX23" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BY23" t="str">
+        <x:v>2.9245584275987415</x:v>
+      </x:c>
+      <x:c r="BZ23" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA23" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB23" t="str">
+        <x:v>east</x:v>
+      </x:c>
+      <x:c r="CC23" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD23" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE23" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF23" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG23" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="30" hidden="0" customHeight="1">
       <x:c r="A24" s="16" t="str">
@@ -13954,6 +15125,52 @@
       </x:c>
       <x:c r="BQ24" s="209" t="str">
         <x:v>H</x:v>
+      </x:c>
+      <x:c r="BR24" t="str">
+        <x:v>TNDC-023</x:v>
+      </x:c>
+      <x:c r="BS24" t="str">
+        <x:v>TN5K-2596</x:v>
+      </x:c>
+      <x:c r="BT24" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BU24" t="str"/>
+      <x:c r="BV24" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BW24" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX24" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BY24" t="str">
+        <x:v>0.6942308247089386</x:v>
+      </x:c>
+      <x:c r="BZ24" t="str">
+        <x:v>nonmetro</x:v>
+      </x:c>
+      <x:c r="CA24" t="str">
+        <x:v>nonmetro_proxy</x:v>
+      </x:c>
+      <x:c r="CB24" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="CC24" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD24" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE24" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF24" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG24" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="30" hidden="0" customHeight="1">
@@ -14154,6 +15371,54 @@
       <x:c r="BQ25" s="209" t="str">
         <x:v>H</x:v>
       </x:c>
+      <x:c r="BR25" t="str">
+        <x:v>TNDC-024</x:v>
+      </x:c>
+      <x:c r="BS25" t="str">
+        <x:v>TN5K-2669</x:v>
+      </x:c>
+      <x:c r="BT25" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU25" t="str">
+        <x:v>regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV25" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BW25" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX25" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY25" t="str">
+        <x:v>0.9771514700518714</x:v>
+      </x:c>
+      <x:c r="BZ25" t="str">
+        <x:v>nonmetro</x:v>
+      </x:c>
+      <x:c r="CA25" t="str">
+        <x:v>nonmetro_proxy</x:v>
+      </x:c>
+      <x:c r="CB25" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="CC25" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD25" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE25" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF25" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG25" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="30" hidden="0" customHeight="1">
       <x:c r="A26" s="16" t="str">
@@ -14355,6 +15620,54 @@
       <x:c r="BQ26" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR26" t="str">
+        <x:v>TNDC-026</x:v>
+      </x:c>
+      <x:c r="BS26" t="str">
+        <x:v>TN5K-0096</x:v>
+      </x:c>
+      <x:c r="BT26" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU26" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV26" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW26" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX26" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY26" t="str">
+        <x:v>0.3144090523322423</x:v>
+      </x:c>
+      <x:c r="BZ26" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA26" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB26" t="str">
+        <x:v>west</x:v>
+      </x:c>
+      <x:c r="CC26" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD26" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE26" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF26" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG26" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="30" hidden="0" customHeight="1">
       <x:c r="A27" s="16" t="str">
@@ -14554,6 +15867,54 @@
       <x:c r="BQ27" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR27" t="str">
+        <x:v>TNDC-027</x:v>
+      </x:c>
+      <x:c r="BS27" t="str">
+        <x:v>TN5K-0074</x:v>
+      </x:c>
+      <x:c r="BT27" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU27" t="str">
+        <x:v>regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV27" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BW27" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX27" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY27" t="str">
+        <x:v>0.3746739998459816</x:v>
+      </x:c>
+      <x:c r="BZ27" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA27" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB27" t="str">
+        <x:v>west</x:v>
+      </x:c>
+      <x:c r="CC27" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD27" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE27" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF27" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG27" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="30" hidden="0" customHeight="1">
       <x:c r="A28" s="16" t="str">
@@ -14758,6 +16119,54 @@
       </x:c>
       <x:c r="BQ28" s="209" t="str">
         <x:v>G</x:v>
+      </x:c>
+      <x:c r="BR28" t="str">
+        <x:v>TNDC-028</x:v>
+      </x:c>
+      <x:c r="BS28" t="str">
+        <x:v>TN5K-0113</x:v>
+      </x:c>
+      <x:c r="BT28" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU28" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV28" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW28" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX28" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY28" t="str">
+        <x:v>0.3547260786096255</x:v>
+      </x:c>
+      <x:c r="BZ28" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA28" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB28" t="str">
+        <x:v>west</x:v>
+      </x:c>
+      <x:c r="CC28" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD28" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE28" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF28" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG28" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="30" hidden="0" customHeight="1">
@@ -14958,6 +16367,54 @@
       <x:c r="BQ29" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR29" t="str">
+        <x:v>TNDC-029</x:v>
+      </x:c>
+      <x:c r="BS29" t="str">
+        <x:v>TN5K-0057</x:v>
+      </x:c>
+      <x:c r="BT29" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU29" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV29" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW29" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX29" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY29" t="str">
+        <x:v>0.3518414778841866</x:v>
+      </x:c>
+      <x:c r="BZ29" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA29" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB29" t="str">
+        <x:v>west</x:v>
+      </x:c>
+      <x:c r="CC29" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD29" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE29" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF29" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG29" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="30" hidden="0" customHeight="1">
       <x:c r="A30" s="16" t="str">
@@ -15159,6 +16616,54 @@
       <x:c r="BQ30" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR30" t="str">
+        <x:v>TNDC-030</x:v>
+      </x:c>
+      <x:c r="BS30" t="str">
+        <x:v>TN5K-0007</x:v>
+      </x:c>
+      <x:c r="BT30" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU30" t="str">
+        <x:v>open_water;protected_land</x:v>
+      </x:c>
+      <x:c r="BV30" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW30" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BX30" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BY30" t="str">
+        <x:v>0.13380941024257076</x:v>
+      </x:c>
+      <x:c r="BZ30" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA30" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB30" t="str">
+        <x:v>west</x:v>
+      </x:c>
+      <x:c r="CC30" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD30" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE30" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF30" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG30" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="30" hidden="0" customHeight="1">
       <x:c r="A31" s="16" t="str">
@@ -15363,6 +16868,34 @@
       </x:c>
       <x:c r="BQ31" s="209" t="str">
         <x:v>G</x:v>
+      </x:c>
+      <x:c r="BR31" t="str">
+        <x:v>TNDC-031</x:v>
+      </x:c>
+      <x:c r="BS31" t="str"/>
+      <x:c r="BT31" t="str"/>
+      <x:c r="BU31" t="str"/>
+      <x:c r="BV31" t="str"/>
+      <x:c r="BW31" t="str"/>
+      <x:c r="BX31" t="str"/>
+      <x:c r="BY31" t="str"/>
+      <x:c r="BZ31" t="str"/>
+      <x:c r="CA31" t="str"/>
+      <x:c r="CB31" t="str"/>
+      <x:c r="CC31" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD31" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE31" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF31" t="str">
+        <x:v>not_mappable</x:v>
+      </x:c>
+      <x:c r="CG31" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="30" hidden="0" customHeight="1">
@@ -15566,6 +17099,54 @@
       </x:c>
       <x:c r="BQ32" s="209" t="str">
         <x:v>G</x:v>
+      </x:c>
+      <x:c r="BR32" t="str">
+        <x:v>TNDC-032</x:v>
+      </x:c>
+      <x:c r="BS32" t="str">
+        <x:v>TN5K-1969</x:v>
+      </x:c>
+      <x:c r="BT32" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU32" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV32" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW32" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX32" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY32" t="str">
+        <x:v>1.356198446618186</x:v>
+      </x:c>
+      <x:c r="BZ32" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA32" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB32" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="CC32" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD32" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE32" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF32" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG32" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="30" hidden="0" customHeight="1">
@@ -15766,6 +17347,54 @@
       <x:c r="BQ33" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR33" t="str">
+        <x:v>TNDC-033</x:v>
+      </x:c>
+      <x:c r="BS33" t="str">
+        <x:v>TN5K-2008</x:v>
+      </x:c>
+      <x:c r="BT33" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU33" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV33" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW33" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX33" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY33" t="str">
+        <x:v>0.9650822447405921</x:v>
+      </x:c>
+      <x:c r="BZ33" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA33" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB33" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="CC33" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD33" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE33" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF33" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG33" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="30" hidden="0" customHeight="1">
       <x:c r="A34" s="16" t="str">
@@ -15968,6 +17597,54 @@
       </x:c>
       <x:c r="BQ34" s="209" t="str">
         <x:v>G</x:v>
+      </x:c>
+      <x:c r="BR34" t="str">
+        <x:v>TNDC-034</x:v>
+      </x:c>
+      <x:c r="BS34" t="str">
+        <x:v>TN5K-1971</x:v>
+      </x:c>
+      <x:c r="BT34" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU34" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV34" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW34" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX34" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY34" t="str">
+        <x:v>0.9799223012394376</x:v>
+      </x:c>
+      <x:c r="BZ34" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA34" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB34" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="CC34" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD34" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE34" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF34" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG34" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="30" hidden="0" customHeight="1">
@@ -16170,6 +17847,54 @@
       <x:c r="BQ35" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR35" t="str">
+        <x:v>TNDC-035</x:v>
+      </x:c>
+      <x:c r="BS35" t="str">
+        <x:v>TN5K-1971</x:v>
+      </x:c>
+      <x:c r="BT35" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU35" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV35" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW35" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX35" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY35" t="str">
+        <x:v>0.9799223012394376</x:v>
+      </x:c>
+      <x:c r="BZ35" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA35" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB35" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="CC35" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD35" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE35" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF35" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG35" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="30" hidden="0" customHeight="1">
       <x:c r="A36" s="16" t="str">
@@ -16369,6 +18094,54 @@
       <x:c r="BQ36" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR36" t="str">
+        <x:v>TNDC-036</x:v>
+      </x:c>
+      <x:c r="BS36" t="str">
+        <x:v>TN5K-1933</x:v>
+      </x:c>
+      <x:c r="BT36" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU36" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV36" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW36" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX36" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY36" t="str">
+        <x:v>1.0332035091188219</x:v>
+      </x:c>
+      <x:c r="BZ36" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA36" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB36" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="CC36" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD36" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE36" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF36" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG36" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="30" hidden="0" customHeight="1">
       <x:c r="A37" s="16" t="str">
@@ -16568,6 +18341,54 @@
       <x:c r="BQ37" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR37" t="str">
+        <x:v>TNDC-037</x:v>
+      </x:c>
+      <x:c r="BS37" t="str">
+        <x:v>TN5K-1970</x:v>
+      </x:c>
+      <x:c r="BT37" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU37" t="str">
+        <x:v>regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV37" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BW37" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX37" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY37" t="str">
+        <x:v>0.9010956386725107</x:v>
+      </x:c>
+      <x:c r="BZ37" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA37" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB37" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="CC37" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD37" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE37" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF37" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG37" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="30" hidden="0" customHeight="1">
       <x:c r="A38" s="16" t="str">
@@ -16767,6 +18588,54 @@
       <x:c r="BQ38" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR38" t="str">
+        <x:v>TNDC-038</x:v>
+      </x:c>
+      <x:c r="BS38" t="str">
+        <x:v>TN5K-2044</x:v>
+      </x:c>
+      <x:c r="BT38" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU38" t="str">
+        <x:v>open_water;protected_land;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV38" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW38" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BX38" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY38" t="str">
+        <x:v>1.0770922071403928</x:v>
+      </x:c>
+      <x:c r="BZ38" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA38" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB38" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="CC38" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD38" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE38" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF38" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG38" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="30" hidden="0" customHeight="1">
       <x:c r="A39" s="16" t="str">
@@ -16969,6 +18838,54 @@
       </x:c>
       <x:c r="BQ39" s="209" t="str">
         <x:v>G</x:v>
+      </x:c>
+      <x:c r="BR39" t="str">
+        <x:v>TNDC-039</x:v>
+      </x:c>
+      <x:c r="BS39" t="str">
+        <x:v>TN5K-1933</x:v>
+      </x:c>
+      <x:c r="BT39" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU39" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV39" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW39" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX39" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY39" t="str">
+        <x:v>1.0332035091188219</x:v>
+      </x:c>
+      <x:c r="BZ39" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA39" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB39" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="CC39" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD39" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE39" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF39" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG39" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="30" hidden="0" customHeight="1">
@@ -17170,6 +19087,54 @@
       </x:c>
       <x:c r="BQ40" s="209" t="str">
         <x:v>G</x:v>
+      </x:c>
+      <x:c r="BR40" t="str">
+        <x:v>TNDC-040</x:v>
+      </x:c>
+      <x:c r="BS40" t="str">
+        <x:v>TN5K-1935</x:v>
+      </x:c>
+      <x:c r="BT40" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU40" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV40" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW40" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX40" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY40" t="str">
+        <x:v>2.057216021749708</x:v>
+      </x:c>
+      <x:c r="BZ40" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA40" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB40" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="CC40" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD40" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE40" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF40" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG40" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="30" hidden="0" customHeight="1">
@@ -17370,6 +19335,54 @@
       <x:c r="BQ41" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR41" t="str">
+        <x:v>TNDC-041</x:v>
+      </x:c>
+      <x:c r="BS41" t="str">
+        <x:v>TN5K-1971</x:v>
+      </x:c>
+      <x:c r="BT41" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU41" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV41" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW41" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX41" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY41" t="str">
+        <x:v>0.9799223012394376</x:v>
+      </x:c>
+      <x:c r="BZ41" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA41" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB41" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="CC41" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD41" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE41" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF41" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG41" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="30" hidden="0" customHeight="1">
       <x:c r="A42" s="16" t="str">
@@ -17569,6 +19582,54 @@
       <x:c r="BQ42" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR42" t="str">
+        <x:v>TNDC-042</x:v>
+      </x:c>
+      <x:c r="BS42" t="str">
+        <x:v>TN5K-1971</x:v>
+      </x:c>
+      <x:c r="BT42" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU42" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV42" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW42" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX42" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY42" t="str">
+        <x:v>0.9799223012394376</x:v>
+      </x:c>
+      <x:c r="BZ42" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA42" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB42" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="CC42" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD42" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE42" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF42" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG42" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="30" hidden="0" customHeight="1">
       <x:c r="A43" s="16" t="str">
@@ -17769,6 +19830,52 @@
       </x:c>
       <x:c r="BQ43" s="209" t="str">
         <x:v>G</x:v>
+      </x:c>
+      <x:c r="BR43" t="str">
+        <x:v>TNDC-043</x:v>
+      </x:c>
+      <x:c r="BS43" t="str">
+        <x:v>TN5K-3947</x:v>
+      </x:c>
+      <x:c r="BT43" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BU43" t="str"/>
+      <x:c r="BV43" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BW43" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX43" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BY43" t="str">
+        <x:v>1.518314156267378</x:v>
+      </x:c>
+      <x:c r="BZ43" t="str">
+        <x:v>nonmetro</x:v>
+      </x:c>
+      <x:c r="CA43" t="str">
+        <x:v>nonmetro_proxy</x:v>
+      </x:c>
+      <x:c r="CB43" t="str">
+        <x:v>east</x:v>
+      </x:c>
+      <x:c r="CC43" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD43" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE43" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF43" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG43" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="30" hidden="0" customHeight="1">
@@ -17965,6 +20072,54 @@
       <x:c r="BQ44" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR44" t="str">
+        <x:v>TNDC-044</x:v>
+      </x:c>
+      <x:c r="BS44" t="str">
+        <x:v>TN5K-3433</x:v>
+      </x:c>
+      <x:c r="BT44" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU44" t="str">
+        <x:v>open_water</x:v>
+      </x:c>
+      <x:c r="BV44" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW44" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX44" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BY44" t="str">
+        <x:v>1.476711803012424</x:v>
+      </x:c>
+      <x:c r="BZ44" t="str">
+        <x:v>nonmetro</x:v>
+      </x:c>
+      <x:c r="CA44" t="str">
+        <x:v>nonmetro_proxy</x:v>
+      </x:c>
+      <x:c r="CB44" t="str">
+        <x:v>east</x:v>
+      </x:c>
+      <x:c r="CC44" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD44" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE44" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF44" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG44" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="30" hidden="0" customHeight="1">
       <x:c r="A45" s="16" t="str">
@@ -18164,6 +20319,52 @@
       <x:c r="BQ45" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR45" t="str">
+        <x:v>TNDC-045</x:v>
+      </x:c>
+      <x:c r="BS45" t="str">
+        <x:v>TN5K-3471</x:v>
+      </x:c>
+      <x:c r="BT45" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BU45" t="str"/>
+      <x:c r="BV45" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BW45" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX45" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BY45" t="str">
+        <x:v>2.650047527419196</x:v>
+      </x:c>
+      <x:c r="BZ45" t="str">
+        <x:v>nonmetro</x:v>
+      </x:c>
+      <x:c r="CA45" t="str">
+        <x:v>nonmetro_proxy</x:v>
+      </x:c>
+      <x:c r="CB45" t="str">
+        <x:v>east</x:v>
+      </x:c>
+      <x:c r="CC45" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD45" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE45" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF45" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG45" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="30" hidden="0" customHeight="1">
       <x:c r="A46" s="19" t="str">
@@ -18363,6 +20564,54 @@
       <x:c r="BQ46" s="209" t="str">
         <x:v>H</x:v>
       </x:c>
+      <x:c r="BR46" t="str">
+        <x:v>TNDC-046</x:v>
+      </x:c>
+      <x:c r="BS46" t="str">
+        <x:v>TN5K-3642</x:v>
+      </x:c>
+      <x:c r="BT46" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU46" t="str">
+        <x:v>open_water;protected_land;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV46" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW46" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BX46" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY46" t="str">
+        <x:v>1.407417549027337</x:v>
+      </x:c>
+      <x:c r="BZ46" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA46" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB46" t="str">
+        <x:v>east</x:v>
+      </x:c>
+      <x:c r="CC46" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD46" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE46" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF46" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG46" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" t="str">
@@ -18563,6 +20812,54 @@
       </x:c>
       <x:c r="BQ47" s="209" t="str">
         <x:v>G</x:v>
+      </x:c>
+      <x:c r="BR47" t="str">
+        <x:v>TNDC-047</x:v>
+      </x:c>
+      <x:c r="BS47" t="str">
+        <x:v>TN5K-3835</x:v>
+      </x:c>
+      <x:c r="BT47" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU47" t="str">
+        <x:v>protected_land;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV47" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BW47" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BX47" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY47" t="str">
+        <x:v>1.6440967056486342</x:v>
+      </x:c>
+      <x:c r="BZ47" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA47" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB47" t="str">
+        <x:v>east</x:v>
+      </x:c>
+      <x:c r="CC47" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD47" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE47" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF47" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG47" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -18763,6 +21060,54 @@
       <x:c r="BQ48" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR48" t="str">
+        <x:v>TNDC-048</x:v>
+      </x:c>
+      <x:c r="BS48" t="str">
+        <x:v>TN5K-3714</x:v>
+      </x:c>
+      <x:c r="BT48" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU48" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV48" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW48" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX48" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY48" t="str">
+        <x:v>1.3213139159811869</x:v>
+      </x:c>
+      <x:c r="BZ48" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA48" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB48" t="str">
+        <x:v>east</x:v>
+      </x:c>
+      <x:c r="CC48" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD48" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE48" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF48" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG48" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" t="str">
@@ -18962,6 +21307,54 @@
       <x:c r="BQ49" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR49" t="str">
+        <x:v>TNDC-049</x:v>
+      </x:c>
+      <x:c r="BS49" t="str">
+        <x:v>TN5K-3713</x:v>
+      </x:c>
+      <x:c r="BT49" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU49" t="str">
+        <x:v>regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV49" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BW49" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX49" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY49" t="str">
+        <x:v>1.4333170387479994</x:v>
+      </x:c>
+      <x:c r="BZ49" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA49" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB49" t="str">
+        <x:v>east</x:v>
+      </x:c>
+      <x:c r="CC49" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD49" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE49" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF49" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG49" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" t="str">
@@ -19161,6 +21554,54 @@
       <x:c r="BQ50" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR50" t="str">
+        <x:v>TNDC-050</x:v>
+      </x:c>
+      <x:c r="BS50" t="str">
+        <x:v>TN5K-0658</x:v>
+      </x:c>
+      <x:c r="BT50" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU50" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV50" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW50" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX50" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY50" t="str">
+        <x:v>0.6738849745856391</x:v>
+      </x:c>
+      <x:c r="BZ50" t="str">
+        <x:v>nonmetro</x:v>
+      </x:c>
+      <x:c r="CA50" t="str">
+        <x:v>nonmetro_proxy</x:v>
+      </x:c>
+      <x:c r="CB50" t="str">
+        <x:v>west</x:v>
+      </x:c>
+      <x:c r="CC50" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD50" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE50" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF50" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG50" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" t="str">
@@ -19364,6 +21805,54 @@
       <x:c r="BQ51" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR51" t="str">
+        <x:v>TNDC-051</x:v>
+      </x:c>
+      <x:c r="BS51" t="str">
+        <x:v>TN5K-3103</x:v>
+      </x:c>
+      <x:c r="BT51" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU51" t="str">
+        <x:v>open_water;protected_land</x:v>
+      </x:c>
+      <x:c r="BV51" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW51" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BX51" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BY51" t="str">
+        <x:v>1.1300574723217223</x:v>
+      </x:c>
+      <x:c r="BZ51" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA51" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB51" t="str">
+        <x:v>east</x:v>
+      </x:c>
+      <x:c r="CC51" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD51" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE51" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF51" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG51" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" t="str">
@@ -19567,6 +22056,54 @@
       <x:c r="BQ52" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR52" t="str">
+        <x:v>TNDC-052</x:v>
+      </x:c>
+      <x:c r="BS52" t="str">
+        <x:v>TN5K-2224</x:v>
+      </x:c>
+      <x:c r="BT52" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU52" t="str">
+        <x:v>regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV52" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BW52" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX52" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY52" t="str">
+        <x:v>0.23121336433622572</x:v>
+      </x:c>
+      <x:c r="BZ52" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA52" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB52" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="CC52" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD52" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE52" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF52" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG52" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" t="str">
@@ -19768,6 +22305,54 @@
       <x:c r="BQ53" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR53" t="str">
+        <x:v>TNDC-053</x:v>
+      </x:c>
+      <x:c r="BS53" t="str">
+        <x:v>TN5K-1930</x:v>
+      </x:c>
+      <x:c r="BT53" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU53" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV53" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW53" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX53" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY53" t="str">
+        <x:v>2.160529683033625</x:v>
+      </x:c>
+      <x:c r="BZ53" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA53" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB53" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="CC53" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD53" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE53" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF53" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG53" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" t="str">
@@ -19969,6 +22554,54 @@
       <x:c r="BQ54" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR54" t="str">
+        <x:v>TNDC-054</x:v>
+      </x:c>
+      <x:c r="BS54" t="str">
+        <x:v>TN5K-2008</x:v>
+      </x:c>
+      <x:c r="BT54" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU54" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV54" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW54" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX54" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY54" t="str">
+        <x:v>0.9650822447405921</x:v>
+      </x:c>
+      <x:c r="BZ54" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA54" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB54" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="CC54" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD54" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE54" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF54" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG54" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" t="str">
@@ -20170,6 +22803,54 @@
       <x:c r="BQ55" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR55" t="str">
+        <x:v>TNDC-055</x:v>
+      </x:c>
+      <x:c r="BS55" t="str">
+        <x:v>TN5K-1970</x:v>
+      </x:c>
+      <x:c r="BT55" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU55" t="str">
+        <x:v>regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV55" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BW55" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX55" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY55" t="str">
+        <x:v>0.9010956386725107</x:v>
+      </x:c>
+      <x:c r="BZ55" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA55" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB55" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="CC55" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD55" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE55" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF55" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG55" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" t="str">
@@ -20372,6 +23053,54 @@
       </x:c>
       <x:c r="BQ56" s="209" t="str">
         <x:v>G</x:v>
+      </x:c>
+      <x:c r="BR56" t="str">
+        <x:v>TNDC-056</x:v>
+      </x:c>
+      <x:c r="BS56" t="str">
+        <x:v>TN5K-1970</x:v>
+      </x:c>
+      <x:c r="BT56" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU56" t="str">
+        <x:v>regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV56" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BW56" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX56" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY56" t="str">
+        <x:v>0.9010956386725107</x:v>
+      </x:c>
+      <x:c r="BZ56" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA56" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB56" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="CC56" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD56" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE56" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF56" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG56" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -20572,6 +23301,54 @@
       <x:c r="BQ57" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR57" t="str">
+        <x:v>TNDC-057</x:v>
+      </x:c>
+      <x:c r="BS57" t="str">
+        <x:v>TN5K-0076</x:v>
+      </x:c>
+      <x:c r="BT57" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU57" t="str">
+        <x:v>open_water;protected_land;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV57" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW57" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BX57" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY57" t="str">
+        <x:v>0.37594464669624966</x:v>
+      </x:c>
+      <x:c r="BZ57" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA57" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB57" t="str">
+        <x:v>west</x:v>
+      </x:c>
+      <x:c r="CC57" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD57" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE57" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF57" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG57" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" t="str">
@@ -20773,6 +23550,54 @@
       <x:c r="BQ58" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR58" t="str">
+        <x:v>TNDC-058</x:v>
+      </x:c>
+      <x:c r="BS58" t="str">
+        <x:v>TN5K-0074</x:v>
+      </x:c>
+      <x:c r="BT58" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU58" t="str">
+        <x:v>regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV58" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BW58" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX58" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY58" t="str">
+        <x:v>0.3746739998459816</x:v>
+      </x:c>
+      <x:c r="BZ58" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA58" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB58" t="str">
+        <x:v>west</x:v>
+      </x:c>
+      <x:c r="CC58" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD58" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE58" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF58" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG58" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" t="str">
@@ -20975,6 +23800,54 @@
       </x:c>
       <x:c r="BQ59" s="209" t="str">
         <x:v>G</x:v>
+      </x:c>
+      <x:c r="BR59" t="str">
+        <x:v>TNDC-059</x:v>
+      </x:c>
+      <x:c r="BS59" t="str">
+        <x:v>TN5K-0057</x:v>
+      </x:c>
+      <x:c r="BT59" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU59" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV59" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW59" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX59" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY59" t="str">
+        <x:v>0.3518414778841866</x:v>
+      </x:c>
+      <x:c r="BZ59" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA59" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB59" t="str">
+        <x:v>west</x:v>
+      </x:c>
+      <x:c r="CC59" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD59" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE59" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF59" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG59" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -21179,6 +24052,54 @@
       <x:c r="BQ60" s="209" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="BR60" t="str">
+        <x:v>TNDC-060</x:v>
+      </x:c>
+      <x:c r="BS60" t="str">
+        <x:v>TN5K-0077</x:v>
+      </x:c>
+      <x:c r="BT60" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU60" t="str">
+        <x:v>open_water;protected_land;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV60" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW60" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BX60" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY60" t="str">
+        <x:v>0.2519831077920066</x:v>
+      </x:c>
+      <x:c r="BZ60" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="CA60" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="CB60" t="str">
+        <x:v>west</x:v>
+      </x:c>
+      <x:c r="CC60" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD60" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE60" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF60" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG60" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="61">
       <x:c r="A61" t="str">
@@ -21380,6 +24301,54 @@
       <x:c r="BQ61" s="209" t="str">
         <x:v>H</x:v>
       </x:c>
+      <x:c r="BR61" t="str">
+        <x:v>TNDC-061</x:v>
+      </x:c>
+      <x:c r="BS61" t="str">
+        <x:v>TN5K-0594</x:v>
+      </x:c>
+      <x:c r="BT61" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU61" t="str">
+        <x:v>protected_land;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV61" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BW61" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BX61" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY61" t="str">
+        <x:v>0.30347856506705284</x:v>
+      </x:c>
+      <x:c r="BZ61" t="str">
+        <x:v>nonmetro</x:v>
+      </x:c>
+      <x:c r="CA61" t="str">
+        <x:v>nonmetro_proxy</x:v>
+      </x:c>
+      <x:c r="CB61" t="str">
+        <x:v>west</x:v>
+      </x:c>
+      <x:c r="CC61" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD61" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE61" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF61" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG61" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" t="str">
@@ -21584,6 +24553,54 @@
       </x:c>
       <x:c r="BQ62" s="209" t="str">
         <x:v>G</x:v>
+      </x:c>
+      <x:c r="BR62" t="str">
+        <x:v>TNDC-062</x:v>
+      </x:c>
+      <x:c r="BS62" t="str">
+        <x:v>TN5K-4417</x:v>
+      </x:c>
+      <x:c r="BT62" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BU62" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BV62" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BW62" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BX62" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BY62" t="str">
+        <x:v>1.3089620272318523</x:v>
+      </x:c>
+      <x:c r="BZ62" t="str">
+        <x:v>nonmetro</x:v>
+      </x:c>
+      <x:c r="CA62" t="str">
+        <x:v>nonmetro_proxy</x:v>
+      </x:c>
+      <x:c r="CB62" t="str">
+        <x:v>east</x:v>
+      </x:c>
+      <x:c r="CC62" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CD62" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CE62" t="str">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="CF62" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="CG62" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -21644,7 +24661,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc26811007a54dd5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93c813e2fcf143ce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -42507,7 +45524,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3e8f7d618ce4d76"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cd57382c1b4424f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -44549,7 +47566,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d25c43b0a85430e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2f7eb29274f4c41"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -44729,7 +47746,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a11a23e9dcc4dac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R382e68194b2f4993"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -45105,7 +48122,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc738802101c448b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb98e9fcef35f4beb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -45290,7 +48307,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33cb1e09435e4ce0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R898d95e465624112"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -45498,6 +48515,54 @@
       <x:c r="AW1" s="225" t="str">
         <x:v>professional_scientific_employment_flag</x:v>
       </x:c>
+      <x:c r="AX1" s="233" t="str">
+        <x:v>phase2_site_id</x:v>
+      </x:c>
+      <x:c r="AY1" s="233" t="str">
+        <x:v>phase2_domain_cell_id</x:v>
+      </x:c>
+      <x:c r="AZ1" s="233" t="str">
+        <x:v>phase2_d1_feasible</x:v>
+      </x:c>
+      <x:c r="BA1" s="233" t="str">
+        <x:v>phase2_d1_exclusion_reason</x:v>
+      </x:c>
+      <x:c r="BB1" s="233" t="str">
+        <x:v>phase2_open_water_flag</x:v>
+      </x:c>
+      <x:c r="BC1" s="233" t="str">
+        <x:v>phase2_protected_land_flag</x:v>
+      </x:c>
+      <x:c r="BD1" s="233" t="str">
+        <x:v>phase2_regulatory_floodway_flag</x:v>
+      </x:c>
+      <x:c r="BE1" s="233" t="str">
+        <x:v>phase2_mean_slope_deg</x:v>
+      </x:c>
+      <x:c r="BF1" s="233" t="str">
+        <x:v>phase2_urban_context</x:v>
+      </x:c>
+      <x:c r="BG1" s="233" t="str">
+        <x:v>phase2_developed_context</x:v>
+      </x:c>
+      <x:c r="BH1" s="233" t="str">
+        <x:v>phase2_grand_region</x:v>
+      </x:c>
+      <x:c r="BI1" s="233" t="str">
+        <x:v>phase2_primary_weight</x:v>
+      </x:c>
+      <x:c r="BJ1" s="233" t="str">
+        <x:v>phase2_weighted_weight</x:v>
+      </x:c>
+      <x:c r="BK1" s="233" t="str">
+        <x:v>phase2_strict_weight</x:v>
+      </x:c>
+      <x:c r="BL1" s="233" t="str">
+        <x:v>phase2_feature_status</x:v>
+      </x:c>
+      <x:c r="BM1" s="233" t="str">
+        <x:v>phase2_evidence_urls</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="85" t="str">
@@ -45645,6 +48710,54 @@
       <x:c r="AW2" s="226" t="str">
         <x:v>H</x:v>
       </x:c>
+      <x:c r="AX2" t="str">
+        <x:v>TNCAND-002</x:v>
+      </x:c>
+      <x:c r="AY2" t="str">
+        <x:v>TN5K-3569</x:v>
+      </x:c>
+      <x:c r="AZ2" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BA2" t="str">
+        <x:v>protected_land;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BB2" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BC2" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BD2" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BE2" t="str">
+        <x:v>2.2577022512753806</x:v>
+      </x:c>
+      <x:c r="BF2" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="BG2" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="BH2" t="str">
+        <x:v>east</x:v>
+      </x:c>
+      <x:c r="BI2" t="str">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="BJ2" t="str">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="BK2" t="str">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="BL2" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="BM2" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="85" t="str">
@@ -45792,6 +48905,54 @@
       <x:c r="AW3" s="226" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="AX3" t="str">
+        <x:v>TNCAND-003</x:v>
+      </x:c>
+      <x:c r="AY3" t="str">
+        <x:v>TN5K-3713</x:v>
+      </x:c>
+      <x:c r="AZ3" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BA3" t="str">
+        <x:v>regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BB3" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BC3" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BD3" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BE3" t="str">
+        <x:v>1.4333170387479994</x:v>
+      </x:c>
+      <x:c r="BF3" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="BG3" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="BH3" t="str">
+        <x:v>east</x:v>
+      </x:c>
+      <x:c r="BI3" t="str">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="BJ3" t="str">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="BK3" t="str">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="BL3" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="BM3" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="85" t="str">
@@ -45939,6 +49100,54 @@
       <x:c r="AW4" s="226" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="AX4" t="str">
+        <x:v>TNCAND-004</x:v>
+      </x:c>
+      <x:c r="AY4" t="str">
+        <x:v>TN5K-0693</x:v>
+      </x:c>
+      <x:c r="AZ4" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BA4" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BB4" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BC4" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BD4" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BE4" t="str">
+        <x:v>0.5780415849553214</x:v>
+      </x:c>
+      <x:c r="BF4" t="str">
+        <x:v>nonmetro</x:v>
+      </x:c>
+      <x:c r="BG4" t="str">
+        <x:v>nonmetro_proxy</x:v>
+      </x:c>
+      <x:c r="BH4" t="str">
+        <x:v>west</x:v>
+      </x:c>
+      <x:c r="BI4" t="str">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="BJ4" t="str">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="BK4" t="str">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="BL4" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="BM4" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="85" t="str">
@@ -46086,6 +49295,54 @@
       <x:c r="AW5" s="226" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="AX5" t="str">
+        <x:v>TNCAND-005</x:v>
+      </x:c>
+      <x:c r="AY5" t="str">
+        <x:v>TN5K-0692</x:v>
+      </x:c>
+      <x:c r="AZ5" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BA5" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BB5" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BC5" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BD5" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BE5" t="str">
+        <x:v>0.56364430156019</x:v>
+      </x:c>
+      <x:c r="BF5" t="str">
+        <x:v>nonmetro</x:v>
+      </x:c>
+      <x:c r="BG5" t="str">
+        <x:v>nonmetro_proxy</x:v>
+      </x:c>
+      <x:c r="BH5" t="str">
+        <x:v>west</x:v>
+      </x:c>
+      <x:c r="BI5" t="str">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="BJ5" t="str">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="BK5" t="str">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="BL5" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="BM5" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
@@ -46229,6 +49486,54 @@
       <x:c r="AW6" s="226" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="AX6" t="str">
+        <x:v>TNCAND-006</x:v>
+      </x:c>
+      <x:c r="AY6" t="str">
+        <x:v>TN5K-1971</x:v>
+      </x:c>
+      <x:c r="AZ6" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BA6" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BB6" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BC6" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BD6" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BE6" t="str">
+        <x:v>0.9799223012394376</x:v>
+      </x:c>
+      <x:c r="BF6" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="BG6" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="BH6" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="BI6" t="str">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="BJ6" t="str">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="BK6" t="str">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="BL6" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="BM6" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
@@ -46376,6 +49681,54 @@
       <x:c r="AW7" s="226" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="AX7" t="str">
+        <x:v>TNCAND-007</x:v>
+      </x:c>
+      <x:c r="AY7" t="str">
+        <x:v>TN5K-2153</x:v>
+      </x:c>
+      <x:c r="AZ7" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BA7" t="str">
+        <x:v>open_water;protected_land;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BB7" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BC7" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BD7" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BE7" t="str">
+        <x:v>0.34054579999711776</x:v>
+      </x:c>
+      <x:c r="BF7" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="BG7" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="BH7" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="BI7" t="str">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="BJ7" t="str">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="BK7" t="str">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="BL7" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="BM7" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
@@ -46523,6 +49876,54 @@
       <x:c r="AW8" s="226" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="AX8" t="str">
+        <x:v>TNCAND-008</x:v>
+      </x:c>
+      <x:c r="AY8" t="str">
+        <x:v>TN5K-1971</x:v>
+      </x:c>
+      <x:c r="AZ8" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BA8" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BB8" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BC8" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BD8" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BE8" t="str">
+        <x:v>0.9799223012394376</x:v>
+      </x:c>
+      <x:c r="BF8" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="BG8" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="BH8" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="BI8" t="str">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="BJ8" t="str">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="BK8" t="str">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="BL8" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="BM8" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
@@ -46668,6 +50069,54 @@
       <x:c r="AW9" s="226" t="str">
         <x:v>H</x:v>
       </x:c>
+      <x:c r="AX9" t="str">
+        <x:v>TNCAND-009</x:v>
+      </x:c>
+      <x:c r="AY9" t="str">
+        <x:v>TN5K-3606</x:v>
+      </x:c>
+      <x:c r="AZ9" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BA9" t="str">
+        <x:v>open_water;protected_land</x:v>
+      </x:c>
+      <x:c r="BB9" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BC9" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BD9" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BE9" t="str">
+        <x:v>1.9046613375345867</x:v>
+      </x:c>
+      <x:c r="BF9" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="BG9" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="BH9" t="str">
+        <x:v>east</x:v>
+      </x:c>
+      <x:c r="BI9" t="str">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="BJ9" t="str">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="BK9" t="str">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="BL9" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="BM9" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
@@ -46815,6 +50264,54 @@
       <x:c r="AW10" s="226" t="str">
         <x:v>H</x:v>
       </x:c>
+      <x:c r="AX10" t="str">
+        <x:v>TNCAND-010</x:v>
+      </x:c>
+      <x:c r="AY10" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="AZ10" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BA10" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BB10" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BC10" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BD10" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BE10" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BF10" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BG10" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BH10" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BI10" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BJ10" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BK10" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BL10" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BM10" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
@@ -46961,6 +50458,54 @@
       </x:c>
       <x:c r="AW11" s="226" t="str">
         <x:v>G</x:v>
+      </x:c>
+      <x:c r="AX11" t="str">
+        <x:v>TNCAND-011</x:v>
+      </x:c>
+      <x:c r="AY11" t="str">
+        <x:v>TN5K-1932</x:v>
+      </x:c>
+      <x:c r="AZ11" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BA11" t="str">
+        <x:v>regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BB11" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BC11" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BD11" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BE11" t="str">
+        <x:v>0.9573106169700623</x:v>
+      </x:c>
+      <x:c r="BF11" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="BG11" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="BH11" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="BI11" t="str">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="BJ11" t="str">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="BK11" t="str">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="BL11" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="BM11" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -47105,6 +50650,54 @@
       <x:c r="AW12" s="226" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="AX12" t="str">
+        <x:v>TNCAND-012</x:v>
+      </x:c>
+      <x:c r="AY12" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="AZ12" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BA12" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BB12" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BC12" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BD12" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BE12" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BF12" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BG12" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BH12" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BI12" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BJ12" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BK12" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BL12" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
+      <x:c r="BM12" t="str">
+        <x:v>not_in_phase2_cohort</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
@@ -47250,6 +50843,54 @@
       <x:c r="AW13" s="226" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="AX13" t="str">
+        <x:v>TNCAND-013</x:v>
+      </x:c>
+      <x:c r="AY13" t="str">
+        <x:v>TN5K-2991</x:v>
+      </x:c>
+      <x:c r="AZ13" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BA13" t="str">
+        <x:v>open_water;protected_land;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BB13" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BC13" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BD13" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BE13" t="str">
+        <x:v>1.550307285454538</x:v>
+      </x:c>
+      <x:c r="BF13" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="BG13" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="BH13" t="str">
+        <x:v>east</x:v>
+      </x:c>
+      <x:c r="BI13" t="str">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="BJ13" t="str">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="BK13" t="str">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="BL13" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="BM13" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
@@ -47397,6 +51038,54 @@
       <x:c r="AW14" s="226" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="AX14" t="str">
+        <x:v>TNCAND-014</x:v>
+      </x:c>
+      <x:c r="AY14" t="str">
+        <x:v>TN5K-1971</x:v>
+      </x:c>
+      <x:c r="AZ14" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BA14" t="str">
+        <x:v>open_water;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BB14" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BC14" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BD14" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BE14" t="str">
+        <x:v>0.9799223012394376</x:v>
+      </x:c>
+      <x:c r="BF14" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="BG14" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="BH14" t="str">
+        <x:v>middle</x:v>
+      </x:c>
+      <x:c r="BI14" t="str">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="BJ14" t="str">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="BK14" t="str">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="BL14" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="BM14" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
@@ -47542,6 +51231,54 @@
       <x:c r="AW15" s="226" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="AX15" t="str">
+        <x:v>TNCAND-015</x:v>
+      </x:c>
+      <x:c r="AY15" t="str">
+        <x:v>TN5K-0076</x:v>
+      </x:c>
+      <x:c r="AZ15" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BA15" t="str">
+        <x:v>open_water;protected_land;regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BB15" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BC15" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BD15" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BE15" t="str">
+        <x:v>0.37594464669624966</x:v>
+      </x:c>
+      <x:c r="BF15" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="BG15" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="BH15" t="str">
+        <x:v>west</x:v>
+      </x:c>
+      <x:c r="BI15" t="str">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="BJ15" t="str">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="BK15" t="str">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="BL15" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="BM15" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
@@ -47687,6 +51424,54 @@
       <x:c r="AW16" s="226" t="str">
         <x:v>G</x:v>
       </x:c>
+      <x:c r="AX16" t="str">
+        <x:v>TNCAND-016</x:v>
+      </x:c>
+      <x:c r="AY16" t="str">
+        <x:v>TN5K-0074</x:v>
+      </x:c>
+      <x:c r="AZ16" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BA16" t="str">
+        <x:v>regulatory_floodway</x:v>
+      </x:c>
+      <x:c r="BB16" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BC16" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BD16" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BE16" t="str">
+        <x:v>0.3746739998459816</x:v>
+      </x:c>
+      <x:c r="BF16" t="str">
+        <x:v>metro_50km</x:v>
+      </x:c>
+      <x:c r="BG16" t="str">
+        <x:v>metro_proxy</x:v>
+      </x:c>
+      <x:c r="BH16" t="str">
+        <x:v>west</x:v>
+      </x:c>
+      <x:c r="BI16" t="str">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="BJ16" t="str">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="BK16" t="str">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="BL16" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="BM16" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">
@@ -47833,6 +51618,52 @@
       </x:c>
       <x:c r="AW17" s="226" t="str">
         <x:v>G</x:v>
+      </x:c>
+      <x:c r="AX17" t="str">
+        <x:v>TNCAND-017</x:v>
+      </x:c>
+      <x:c r="AY17" t="str">
+        <x:v>TN5K-4488</x:v>
+      </x:c>
+      <x:c r="AZ17" t="str">
+        <x:v>True</x:v>
+      </x:c>
+      <x:c r="BA17" t="str"/>
+      <x:c r="BB17" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BC17" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BD17" t="str">
+        <x:v>False</x:v>
+      </x:c>
+      <x:c r="BE17" t="str">
+        <x:v>5.5128147337171765</x:v>
+      </x:c>
+      <x:c r="BF17" t="str">
+        <x:v>nonmetro</x:v>
+      </x:c>
+      <x:c r="BG17" t="str">
+        <x:v>nonmetro_proxy</x:v>
+      </x:c>
+      <x:c r="BH17" t="str">
+        <x:v>east</x:v>
+      </x:c>
+      <x:c r="BI17" t="str">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="BJ17" t="str">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="BK17" t="str">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="BL17" t="str">
+        <x:v>complete</x:v>
+      </x:c>
+      <x:c r="BM17" t="str">
+        <x:v>USGS 3DEP; USGS PAD-US; Tennessee DFIRM; USGS NHD</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -47860,7 +51691,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea7a800858b640b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec46d6693e164d2e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>